<commit_message>
Commit pending local work on InitApp
</commit_message>
<xml_diff>
--- a/WebApp/App_Data/SizingExcels/N2GeneratorSizing.xlsx
+++ b/WebApp/App_Data/SizingExcels/N2GeneratorSizing.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26227"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Uploads\SizingExcels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Havayar\HavayarApp\WebApp\App_Data\SizingExcels\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{535C4486-7412-4710-92ED-1C6C2FC7AA58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="2"/>
+    <workbookView xWindow="3072" yWindow="3072" windowWidth="30960" windowHeight="12120" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipment Selection" sheetId="1" r:id="rId1"/>
@@ -34,7 +35,7 @@
     <definedName name="Oxymat.N2.Generator.Volume">Table3[Adsorbent Volume, Lit]</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">Datasheet!$A$1:$U$48</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -43,6 +44,8 @@
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -1130,7 +1133,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
@@ -2171,17 +2174,20 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -2205,36 +2211,375 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="36" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="5" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="5" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="5" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="9" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="37" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="40" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="41" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="42" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="43" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="44" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="16" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="45" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="46" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="47" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="45" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="6" borderId="45" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="6" borderId="34" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="6" borderId="40" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="6" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="6" borderId="42" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="6" borderId="43" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="6" borderId="44" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="18" fillId="6" borderId="28" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="43" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="44" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="28" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="16" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="7" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="13" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="29" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="0" borderId="26" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="6" borderId="34" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="6" borderId="44" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="17" fillId="6" borderId="28" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="48" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="29" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="29" xfId="4" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="18" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="49" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="11" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="18" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="36" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="16" fillId="0" borderId="6" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="6" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="17" fillId="0" borderId="10" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="18" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="36" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="10" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="36" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="6" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="16" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="16" fillId="0" borderId="7" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="6" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="18" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="16" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="7" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="17" fillId="0" borderId="7" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2244,365 +2589,23 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="13" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="8" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="9" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="37" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="36" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="6" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="10" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="36" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="16" fillId="0" borderId="6" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="18" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="11" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="36" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="6" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="6" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="10" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="18" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="17" fillId="0" borderId="0" xfId="6" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="6" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="6" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="49" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="29" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="0" borderId="26" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="6" borderId="34" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="6" borderId="44" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="17" fillId="6" borderId="28" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="48" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="29" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="29" xfId="4" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="40" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="41" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="42" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="43" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="44" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="16" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="7" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="45" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="46" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="47" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="45" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="6" borderId="45" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="16" fillId="6" borderId="34" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="6" borderId="40" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="6" borderId="41" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="6" borderId="42" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="6" borderId="43" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="6" borderId="44" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="18" fillId="6" borderId="28" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="43" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="44" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="28" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="16" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="7" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="13" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="36" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="36" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="5" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="5" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="37" xfId="5" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
     <cellStyle name="Calculation" xfId="3" builtinId="22"/>
     <cellStyle name="Input" xfId="1" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2 3" xfId="4"/>
-    <cellStyle name="Normal 2 4" xfId="5"/>
-    <cellStyle name="Normal_Linelist" xfId="6"/>
+    <cellStyle name="Normal 2 3" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="Normal 2 4" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="Normal_Linelist" xfId="6" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
     <cellStyle name="Output" xfId="2" builtinId="21"/>
   </cellStyles>
   <dxfs count="13">
@@ -2988,60 +2991,60 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="F50:M64" totalsRowShown="0" dataDxfId="5" tableBorderDxfId="4">
-  <autoFilter ref="F50:M64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="F50:M64" totalsRowShown="0" dataDxfId="5" tableBorderDxfId="4">
+  <autoFilter ref="F50:M64" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" name="N2 Model-Oxymat"/>
-    <tableColumn id="2" name="Adsorbent Volume, Lit">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="N2 Model-Oxymat"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Adsorbent Volume, Lit">
       <calculatedColumnFormula>0.95*Table3[[#This Row],[Towers Net Volume, Lit]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" name="Adsorbent Weight, kg">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Adsorbent Weight, kg">
       <calculatedColumnFormula>Table3[[#This Row],[Adsorbent Volume, Lit]]*0.65</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" name="ID, mm"/>
-    <tableColumn id="5" name="TL-TL, mm"/>
-    <tableColumn id="6" name="Head Factor"/>
-    <tableColumn id="7" name="Towers Net Volume, Lit">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="ID, mm"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="TL-TL, mm"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Head Factor"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Towers Net Volume, Lit">
       <calculatedColumnFormula>2*RIGHT(F51,1)*(PI()/4*Table3[[#This Row],[ID, mm]]^2*Table3[[#This Row],[TL-TL, mm]]+PI()/(6*Table3[[#This Row],[Head Factor]])*Table3[[#This Row],[ID, mm]]^3)/1000000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" name="Generator Dimensions"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Generator Dimensions"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Table6" displayName="Table6" ref="F66:M82" totalsRowShown="0" dataDxfId="2" headerRowBorderDxfId="3" tableBorderDxfId="1" totalsRowBorderDxfId="0">
-  <autoFilter ref="F66:M82"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Table6" displayName="Table6" ref="F66:M82" totalsRowShown="0" dataDxfId="2" headerRowBorderDxfId="3" tableBorderDxfId="1" totalsRowBorderDxfId="0">
+  <autoFilter ref="F66:M82" xr:uid="{00000000-0009-0000-0100-000006000000}"/>
   <tableColumns count="8">
-    <tableColumn id="1" name="N2 Model-Havayar"/>
-    <tableColumn id="2" name="Adsorbent Volume, Lit">
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="N2 Model-Havayar"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Adsorbent Volume, Lit">
       <calculatedColumnFormula>0.95*Table6[[#This Row],[Towers Net Volume, Lit]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" name="Adsorbent Weight, kg">
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Adsorbent Weight, kg">
       <calculatedColumnFormula>Table6[[#This Row],[Adsorbent Volume, Lit]]*0.65</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" name="ID, mm"/>
-    <tableColumn id="5" name="TL-TL, mm"/>
-    <tableColumn id="6" name="Head Factor"/>
-    <tableColumn id="7" name="Towers Net Volume, Lit">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="ID, mm"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="TL-TL, mm"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Head Factor"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="Towers Net Volume, Lit">
       <calculatedColumnFormula>2*RIGHT(F67,1)*(PI()/4*Table6[[#This Row],[ID, mm]]^2*Table6[[#This Row],[TL-TL, mm]]+PI()/(6*Table6[[#This Row],[Head Factor]])*Table6[[#This Row],[ID, mm]]^3)/1000000</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" name="Generator Dimensions"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0100-000008000000}" name="Generator Dimensions"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="Table12" displayName="Table12" ref="F85:G102" totalsRowShown="0">
-  <autoFilter ref="F85:G102"/>
-  <sortState ref="F86:G99">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table12" displayName="Table12" ref="F85:G102" totalsRowShown="0">
+  <autoFilter ref="F85:G102" xr:uid="{00000000-0009-0000-0100-00000C000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="F86:G99">
     <sortCondition descending="1" ref="G86:G99"/>
   </sortState>
   <tableColumns count="2">
-    <tableColumn id="1" name="Model"/>
-    <tableColumn id="2" name="Actual Capacity"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Model"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Actual Capacity"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3309,18 +3312,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M108"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" customWidth="1"/>
-    <col min="2" max="2" width="64.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.33203125" customWidth="1"/>
+    <col min="2" max="2" width="64.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23" bestFit="1" customWidth="1"/>
-    <col min="5" max="12" width="10.7109375" customWidth="1"/>
+    <col min="5" max="12" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="18" t="s">
         <v>67</v>
       </c>
@@ -3333,19 +3336,19 @@
       <c r="D1" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="E1" s="88" t="s">
+      <c r="E1" s="91" t="s">
         <v>64</v>
       </c>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="89"/>
-    </row>
-    <row r="2" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="90" t="s">
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="91"/>
+      <c r="I1" s="91"/>
+      <c r="J1" s="91"/>
+      <c r="K1" s="91"/>
+      <c r="L1" s="92"/>
+    </row>
+    <row r="2" spans="1:12" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="89" t="s">
         <v>100</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -3366,8 +3369,8 @@
       <c r="K2" s="1"/>
       <c r="L2" s="23"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="98"/>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A3" s="99"/>
       <c r="B3" s="1" t="s">
         <v>102</v>
       </c>
@@ -3389,8 +3392,8 @@
       <c r="K3" s="1"/>
       <c r="L3" s="23"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="98"/>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A4" s="99"/>
       <c r="B4" s="1" t="s">
         <v>98</v>
       </c>
@@ -3400,20 +3403,20 @@
       <c r="D4" s="22">
         <v>40</v>
       </c>
-      <c r="E4" s="95" t="str">
+      <c r="E4" s="96" t="str">
         <f>IF(OR(AND(D4&gt;50,D8&lt;=99.99),AND(D4&gt;40,D8&gt;99.99)),"Inlet temperature is too high."," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="F4" s="96"/>
-      <c r="G4" s="96"/>
+      <c r="F4" s="97"/>
+      <c r="G4" s="97"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
       <c r="L4" s="23"/>
     </row>
-    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="98"/>
+    <row r="5" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="99"/>
       <c r="B5" s="14" t="s">
         <v>61</v>
       </c>
@@ -3430,8 +3433,8 @@
       <c r="K5" s="1"/>
       <c r="L5" s="23"/>
     </row>
-    <row r="6" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="91"/>
+    <row r="6" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="90"/>
       <c r="B6" s="16" t="s">
         <v>62</v>
       </c>
@@ -3448,8 +3451,8 @@
       <c r="K6" s="25"/>
       <c r="L6" s="26"/>
     </row>
-    <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="90" t="s">
+    <row r="7" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="89" t="s">
         <v>56</v>
       </c>
       <c r="B7" s="20" t="s">
@@ -3470,8 +3473,8 @@
       <c r="K7" s="20"/>
       <c r="L7" s="21"/>
     </row>
-    <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="98"/>
+    <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="99"/>
       <c r="B8" s="1" t="s">
         <v>51</v>
       </c>
@@ -3493,8 +3496,8 @@
       <c r="K8" s="1"/>
       <c r="L8" s="23"/>
     </row>
-    <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="98"/>
+    <row r="9" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="99"/>
       <c r="B9" s="1" t="s">
         <v>27</v>
       </c>
@@ -3504,20 +3507,20 @@
       <c r="D9" s="22">
         <v>1</v>
       </c>
-      <c r="E9" s="95" t="str">
+      <c r="E9" s="96" t="str">
         <f ca="1">IF(AND(D28="Custom model Required",D8&gt;99.99),"Increase the number of N2 Generators on duty."," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="F9" s="96"/>
-      <c r="G9" s="96"/>
-      <c r="H9" s="96"/>
-      <c r="I9" s="96"/>
+      <c r="F9" s="97"/>
+      <c r="G9" s="97"/>
+      <c r="H9" s="97"/>
+      <c r="I9" s="97"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="23"/>
     </row>
-    <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="98"/>
+    <row r="10" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="99"/>
       <c r="B10" s="1" t="s">
         <v>5</v>
       </c>
@@ -3527,31 +3530,31 @@
       <c r="D10" s="22" t="s">
         <v>263</v>
       </c>
-      <c r="E10" s="95" t="str">
+      <c r="E10" s="96" t="str">
         <f>IF(AND(D10="SHE",D8&gt;99.99),"For High Purity solely select Kurary."," ")</f>
         <v xml:space="preserve"> </v>
       </c>
-      <c r="F10" s="96"/>
-      <c r="G10" s="96"/>
-      <c r="H10" s="96"/>
+      <c r="F10" s="97"/>
+      <c r="G10" s="97"/>
+      <c r="H10" s="97"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="23"/>
     </row>
-    <row r="11" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="91"/>
+    <row r="11" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="90"/>
       <c r="B11" s="25" t="s">
         <v>60</v>
       </c>
       <c r="C11" s="17"/>
-      <c r="D11" s="97" t="s">
+      <c r="D11" s="98" t="s">
         <v>264</v>
       </c>
-      <c r="E11" s="97" t="s">
+      <c r="E11" s="98" t="s">
         <v>264</v>
       </c>
-      <c r="F11" s="97" t="s">
+      <c r="F11" s="98" t="s">
         <v>264</v>
       </c>
       <c r="G11" s="28"/>
@@ -3561,7 +3564,7 @@
       <c r="K11" s="25"/>
       <c r="L11" s="26"/>
     </row>
-    <row r="12" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="48"/>
       <c r="B12" s="25" t="s">
         <v>54</v>
@@ -3582,11 +3585,11 @@
       <c r="K12" s="25"/>
       <c r="L12" s="26"/>
     </row>
-    <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="90" t="s">
+    <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="89" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="93" t="s">
+      <c r="B13" s="94" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="30" t="s">
@@ -3607,9 +3610,9 @@
       <c r="K13" s="20"/>
       <c r="L13" s="21"/>
     </row>
-    <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="98"/>
-      <c r="B14" s="94"/>
+    <row r="14" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="99"/>
+      <c r="B14" s="95"/>
       <c r="C14" s="8" t="s">
         <v>55</v>
       </c>
@@ -3628,8 +3631,8 @@
       <c r="K14" s="1"/>
       <c r="L14" s="23"/>
     </row>
-    <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="98"/>
+    <row r="15" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="99"/>
       <c r="B15" s="34" t="s">
         <v>22</v>
       </c>
@@ -3649,8 +3652,8 @@
       <c r="K15" s="1"/>
       <c r="L15" s="23"/>
     </row>
-    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="98"/>
+    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="99"/>
       <c r="B16" s="1" t="s">
         <v>14</v>
       </c>
@@ -3670,8 +3673,8 @@
       <c r="K16" s="1"/>
       <c r="L16" s="23"/>
     </row>
-    <row r="17" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="98"/>
+    <row r="17" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="99"/>
       <c r="B17" s="1" t="s">
         <v>20</v>
       </c>
@@ -3689,8 +3692,8 @@
       <c r="K17" s="1"/>
       <c r="L17" s="23"/>
     </row>
-    <row r="18" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="98"/>
+    <row r="18" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="99"/>
       <c r="B18" s="1" t="s">
         <v>23</v>
       </c>
@@ -3708,8 +3711,8 @@
       <c r="K18" s="1"/>
       <c r="L18" s="23"/>
     </row>
-    <row r="19" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="98"/>
+    <row r="19" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="99"/>
       <c r="B19" s="1" t="s">
         <v>15</v>
       </c>
@@ -3729,8 +3732,8 @@
       <c r="K19" s="1"/>
       <c r="L19" s="23"/>
     </row>
-    <row r="20" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="98"/>
+    <row r="20" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="99"/>
       <c r="B20" s="1" t="s">
         <v>21</v>
       </c>
@@ -3748,8 +3751,8 @@
       <c r="K20" s="1"/>
       <c r="L20" s="23"/>
     </row>
-    <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="98"/>
+    <row r="21" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="99"/>
       <c r="B21" s="1" t="s">
         <v>24</v>
       </c>
@@ -3767,8 +3770,8 @@
       <c r="K21" s="1"/>
       <c r="L21" s="23"/>
     </row>
-    <row r="22" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="98"/>
+    <row r="22" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="99"/>
       <c r="B22" s="47" t="s">
         <v>86</v>
       </c>
@@ -3785,8 +3788,8 @@
       <c r="K22" s="1"/>
       <c r="L22" s="23"/>
     </row>
-    <row r="23" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="98"/>
+    <row r="23" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="99"/>
       <c r="B23" s="47" t="s">
         <v>88</v>
       </c>
@@ -3804,8 +3807,8 @@
       <c r="K23" s="1"/>
       <c r="L23" s="23"/>
     </row>
-    <row r="24" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="98"/>
+    <row r="24" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="99"/>
       <c r="B24" s="1" t="s">
         <v>31</v>
       </c>
@@ -3826,8 +3829,8 @@
       <c r="K24" s="1"/>
       <c r="L24" s="23"/>
     </row>
-    <row r="25" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="98"/>
+    <row r="25" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="99"/>
       <c r="B25" s="1" t="s">
         <v>87</v>
       </c>
@@ -3847,9 +3850,9 @@
       <c r="K25" s="1"/>
       <c r="L25" s="23"/>
     </row>
-    <row r="26" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="98"/>
-      <c r="B26" s="94" t="s">
+    <row r="26" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="99"/>
+      <c r="B26" s="95" t="s">
         <v>28</v>
       </c>
       <c r="C26" s="1" t="s">
@@ -3868,9 +3871,9 @@
       <c r="K26" s="1"/>
       <c r="L26" s="23"/>
     </row>
-    <row r="27" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="98"/>
-      <c r="B27" s="94"/>
+    <row r="27" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="99"/>
+      <c r="B27" s="95"/>
       <c r="C27" s="1" t="s">
         <v>16</v>
       </c>
@@ -3887,9 +3890,9 @@
       <c r="K27" s="1"/>
       <c r="L27" s="23"/>
     </row>
-    <row r="28" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="98"/>
-      <c r="B28" s="94" t="s">
+    <row r="28" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="99"/>
+      <c r="B28" s="95" t="s">
         <v>82</v>
       </c>
       <c r="C28" s="2" t="s">
@@ -3908,9 +3911,9 @@
       <c r="K28" s="1"/>
       <c r="L28" s="23"/>
     </row>
-    <row r="29" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="98"/>
-      <c r="B29" s="94"/>
+    <row r="29" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="99"/>
+      <c r="B29" s="95"/>
       <c r="C29" s="2" t="s">
         <v>47</v>
       </c>
@@ -3926,8 +3929,8 @@
       <c r="K29" s="1"/>
       <c r="L29" s="23"/>
     </row>
-    <row r="30" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="98"/>
+    <row r="30" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="99"/>
       <c r="B30" s="34" t="s">
         <v>243</v>
       </c>
@@ -3947,8 +3950,8 @@
       <c r="K30" s="1"/>
       <c r="L30" s="23"/>
     </row>
-    <row r="31" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="98"/>
+    <row r="31" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="99"/>
       <c r="B31" s="34" t="s">
         <v>244</v>
       </c>
@@ -3968,8 +3971,8 @@
       <c r="K31" s="1"/>
       <c r="L31" s="23"/>
     </row>
-    <row r="32" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="98"/>
+    <row r="32" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="99"/>
       <c r="B32" s="34" t="s">
         <v>59</v>
       </c>
@@ -3987,8 +3990,8 @@
       <c r="K32" s="1"/>
       <c r="L32" s="23"/>
     </row>
-    <row r="33" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="98"/>
+    <row r="33" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="99"/>
       <c r="B33" s="34" t="s">
         <v>91</v>
       </c>
@@ -4009,8 +4012,8 @@
       <c r="K33" s="1"/>
       <c r="L33" s="23"/>
     </row>
-    <row r="34" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="98"/>
+    <row r="34" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="99"/>
       <c r="B34" s="34" t="s">
         <v>94</v>
       </c>
@@ -4030,8 +4033,8 @@
       <c r="K34" s="1"/>
       <c r="L34" s="23"/>
     </row>
-    <row r="35" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="98"/>
+    <row r="35" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="99"/>
       <c r="B35" s="34" t="s">
         <v>97</v>
       </c>
@@ -4051,8 +4054,8 @@
       <c r="K35" s="1"/>
       <c r="L35" s="23"/>
     </row>
-    <row r="36" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="98"/>
+    <row r="36" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="99"/>
       <c r="B36" s="34" t="s">
         <v>93</v>
       </c>
@@ -4072,8 +4075,8 @@
       <c r="K36" s="1"/>
       <c r="L36" s="23"/>
     </row>
-    <row r="37" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="91"/>
+    <row r="37" spans="1:12" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="90"/>
       <c r="B37" s="39" t="s">
         <v>89</v>
       </c>
@@ -4081,7 +4084,7 @@
         <v>0</v>
       </c>
       <c r="D37" s="40">
-        <f ca="1">D36*D25+D9*IF(D8&lt;=99.99,((0.9*(D19-2.5)*RIGHT(D29,1)*(D35/1000)*273.15)/(273.15+D16))*(1800/55),((D19-3.5)*(D35/1000)*273.15*RIGHT(D29,1)/(273.15+D16))*(1800/110))</f>
+        <f ca="1">D36*D25+D9*IF(D8&lt;=99.99,((0.9*(D19-2.5)*RIGHT(D29,1)*(D35/1000)*273.15)/(273.15+D16))*(1800/55),D19*D35/1000*273.15*RIGHT(D29,1)/(273.15+D16)*(1800/110))</f>
         <v>11.66949762964984</v>
       </c>
       <c r="E37" s="25"/>
@@ -4093,8 +4096,8 @@
       <c r="K37" s="25"/>
       <c r="L37" s="26"/>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A38" s="90" t="s">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A38" s="89" t="s">
         <v>58</v>
       </c>
       <c r="B38" s="13" t="s">
@@ -4116,8 +4119,8 @@
       <c r="K38" s="20"/>
       <c r="L38" s="21"/>
     </row>
-    <row r="39" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="91"/>
+    <row r="39" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="90"/>
       <c r="B39" s="25" t="s">
         <v>92</v>
       </c>
@@ -4138,8 +4141,8 @@
       <c r="K39" s="25"/>
       <c r="L39" s="26"/>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A40" s="90" t="s">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A40" s="89" t="s">
         <v>68</v>
       </c>
       <c r="B40" s="20" t="s">
@@ -4161,8 +4164,8 @@
       <c r="K40" s="20"/>
       <c r="L40" s="21"/>
     </row>
-    <row r="41" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="91"/>
+    <row r="41" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="90"/>
       <c r="B41" s="25" t="s">
         <v>49</v>
       </c>
@@ -4183,27 +4186,27 @@
       <c r="K41" s="25"/>
       <c r="L41" s="26"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D44" s="7"/>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D45" s="7"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D46" s="7"/>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D47" s="7"/>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="D48" s="7"/>
     </row>
-    <row r="49" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:13" x14ac:dyDescent="0.3">
       <c r="D49" s="7"/>
     </row>
-    <row r="50" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:13" x14ac:dyDescent="0.3">
       <c r="D50" s="7"/>
-      <c r="E50" s="99" t="s">
+      <c r="E50" s="88" t="s">
         <v>18</v>
       </c>
       <c r="F50" s="5" t="s">
@@ -4231,8 +4234,8 @@
         <v>260</v>
       </c>
     </row>
-    <row r="51" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="E51" s="99"/>
+    <row r="51" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="E51" s="88"/>
       <c r="F51" s="9" t="s">
         <v>10</v>
       </c>
@@ -4261,8 +4264,8 @@
         <v>259</v>
       </c>
     </row>
-    <row r="52" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="E52" s="99"/>
+    <row r="52" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="E52" s="88"/>
       <c r="F52" s="10" t="s">
         <v>9</v>
       </c>
@@ -4291,10 +4294,10 @@
         <v>257</v>
       </c>
     </row>
-    <row r="53" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B53" s="92"/>
+    <row r="53" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B53" s="93"/>
       <c r="D53" s="7"/>
-      <c r="E53" s="99"/>
+      <c r="E53" s="88"/>
       <c r="F53" s="9" t="s">
         <v>80</v>
       </c>
@@ -4323,10 +4326,10 @@
         <v>258</v>
       </c>
     </row>
-    <row r="54" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B54" s="92"/>
+    <row r="54" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B54" s="93"/>
       <c r="D54" s="7"/>
-      <c r="E54" s="99"/>
+      <c r="E54" s="88"/>
       <c r="F54" s="10" t="s">
         <v>79</v>
       </c>
@@ -4355,10 +4358,10 @@
         <v>256</v>
       </c>
     </row>
-    <row r="55" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B55" s="92"/>
+    <row r="55" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B55" s="93"/>
       <c r="D55" s="7"/>
-      <c r="E55" s="99"/>
+      <c r="E55" s="88"/>
       <c r="F55" s="9" t="s">
         <v>78</v>
       </c>
@@ -4387,10 +4390,10 @@
         <v>255</v>
       </c>
     </row>
-    <row r="56" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B56" s="92"/>
+    <row r="56" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="B56" s="93"/>
       <c r="D56" s="7"/>
-      <c r="E56" s="99"/>
+      <c r="E56" s="88"/>
       <c r="F56" s="10" t="s">
         <v>77</v>
       </c>
@@ -4419,39 +4422,39 @@
         <v>254</v>
       </c>
     </row>
-    <row r="57" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:13" x14ac:dyDescent="0.3">
       <c r="D57" s="7"/>
-      <c r="E57" s="99"/>
+      <c r="E57" s="88"/>
       <c r="F57" s="9" t="s">
         <v>76</v>
       </c>
       <c r="G57" s="10">
         <f>0.95*Table3[[#This Row],[Towers Net Volume, Lit]]</f>
-        <v>618.7178503768456</v>
+        <v>769.01593991647303</v>
       </c>
       <c r="H57" s="10">
         <f>Table3[[#This Row],[Adsorbent Volume, Lit]]*0.65</f>
-        <v>402.16660274494967</v>
+        <v>499.8603609457075</v>
       </c>
       <c r="I57" s="8">
-        <v>496</v>
+        <v>547</v>
       </c>
       <c r="J57" s="8">
-        <v>1520</v>
+        <v>1540</v>
       </c>
       <c r="K57" s="45">
         <v>2</v>
       </c>
       <c r="L57" s="45">
         <f>2*RIGHT(F57,1)*(PI()/4*Table3[[#This Row],[ID, mm]]^2*Table3[[#This Row],[TL-TL, mm]]+PI()/(6*Table3[[#This Row],[Head Factor]])*Table3[[#This Row],[ID, mm]]^3)/1000000</f>
-        <v>651.28194776510065</v>
+        <v>809.49046306997161</v>
       </c>
       <c r="M57" s="45" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="58" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="E58" s="99"/>
+    <row r="58" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="E58" s="88"/>
       <c r="F58" s="10" t="s">
         <v>75</v>
       </c>
@@ -4480,8 +4483,8 @@
         <v>252</v>
       </c>
     </row>
-    <row r="59" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="E59" s="99"/>
+    <row r="59" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="E59" s="88"/>
       <c r="F59" s="9" t="s">
         <v>74</v>
       </c>
@@ -4510,8 +4513,8 @@
         <v>251</v>
       </c>
     </row>
-    <row r="60" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="E60" s="99"/>
+    <row r="60" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="E60" s="88"/>
       <c r="F60" s="10" t="s">
         <v>73</v>
       </c>
@@ -4540,8 +4543,8 @@
         <v>250</v>
       </c>
     </row>
-    <row r="61" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="E61" s="99"/>
+    <row r="61" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="E61" s="88"/>
       <c r="F61" s="9" t="s">
         <v>72</v>
       </c>
@@ -4570,8 +4573,8 @@
         <v>249</v>
       </c>
     </row>
-    <row r="62" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="E62" s="99"/>
+    <row r="62" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="E62" s="88"/>
       <c r="F62" s="10" t="s">
         <v>71</v>
       </c>
@@ -4600,8 +4603,8 @@
         <v>248</v>
       </c>
     </row>
-    <row r="63" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="E63" s="99"/>
+    <row r="63" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="E63" s="88"/>
       <c r="F63" s="9" t="s">
         <v>70</v>
       </c>
@@ -4630,8 +4633,8 @@
         <v>248</v>
       </c>
     </row>
-    <row r="64" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="E64" s="99"/>
+    <row r="64" spans="2:13" x14ac:dyDescent="0.3">
+      <c r="E64" s="88"/>
       <c r="F64" s="10" t="s">
         <v>69</v>
       </c>
@@ -4660,11 +4663,11 @@
         <v>248</v>
       </c>
     </row>
-    <row r="65" spans="5:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="5:13" x14ac:dyDescent="0.3">
       <c r="E65" s="11"/>
     </row>
-    <row r="66" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E66" s="99" t="s">
+    <row r="66" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E66" s="88" t="s">
         <v>19</v>
       </c>
       <c r="F66" s="6" t="s">
@@ -4692,8 +4695,8 @@
         <v>260</v>
       </c>
     </row>
-    <row r="67" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E67" s="99"/>
+    <row r="67" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E67" s="88"/>
       <c r="F67" s="12" t="s">
         <v>242</v>
       </c>
@@ -4720,8 +4723,8 @@
       </c>
       <c r="M67" s="45"/>
     </row>
-    <row r="68" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E68" s="99"/>
+    <row r="68" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E68" s="88"/>
       <c r="F68" s="12" t="s">
         <v>245</v>
       </c>
@@ -4748,8 +4751,8 @@
       </c>
       <c r="M68" s="45"/>
     </row>
-    <row r="69" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E69" s="99"/>
+    <row r="69" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E69" s="88"/>
       <c r="F69" s="12" t="s">
         <v>241</v>
       </c>
@@ -4778,8 +4781,8 @@
         <v>259</v>
       </c>
     </row>
-    <row r="70" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E70" s="99"/>
+    <row r="70" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E70" s="88"/>
       <c r="F70" s="4" t="s">
         <v>240</v>
       </c>
@@ -4808,8 +4811,8 @@
         <v>257</v>
       </c>
     </row>
-    <row r="71" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E71" s="99"/>
+    <row r="71" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E71" s="88"/>
       <c r="F71" s="12" t="s">
         <v>239</v>
       </c>
@@ -4838,8 +4841,8 @@
         <v>258</v>
       </c>
     </row>
-    <row r="72" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E72" s="99"/>
+    <row r="72" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E72" s="88"/>
       <c r="F72" s="4" t="s">
         <v>238</v>
       </c>
@@ -4868,8 +4871,8 @@
         <v>256</v>
       </c>
     </row>
-    <row r="73" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E73" s="99"/>
+    <row r="73" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E73" s="88"/>
       <c r="F73" s="12" t="s">
         <v>237</v>
       </c>
@@ -4898,8 +4901,8 @@
         <v>255</v>
       </c>
     </row>
-    <row r="74" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E74" s="99"/>
+    <row r="74" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E74" s="88"/>
       <c r="F74" s="4" t="s">
         <v>236</v>
       </c>
@@ -4928,8 +4931,8 @@
         <v>254</v>
       </c>
     </row>
-    <row r="75" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E75" s="99"/>
+    <row r="75" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E75" s="88"/>
       <c r="F75" s="12" t="s">
         <v>228</v>
       </c>
@@ -4958,8 +4961,8 @@
         <v>253</v>
       </c>
     </row>
-    <row r="76" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E76" s="99"/>
+    <row r="76" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E76" s="88"/>
       <c r="F76" s="4" t="s">
         <v>235</v>
       </c>
@@ -4988,8 +4991,8 @@
         <v>252</v>
       </c>
     </row>
-    <row r="77" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E77" s="99"/>
+    <row r="77" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E77" s="88"/>
       <c r="F77" s="12" t="s">
         <v>234</v>
       </c>
@@ -5018,8 +5021,8 @@
         <v>251</v>
       </c>
     </row>
-    <row r="78" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E78" s="99"/>
+    <row r="78" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E78" s="88"/>
       <c r="F78" s="4" t="s">
         <v>229</v>
       </c>
@@ -5048,8 +5051,8 @@
         <v>250</v>
       </c>
     </row>
-    <row r="79" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E79" s="99"/>
+    <row r="79" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E79" s="88"/>
       <c r="F79" s="12" t="s">
         <v>232</v>
       </c>
@@ -5078,8 +5081,8 @@
         <v>249</v>
       </c>
     </row>
-    <row r="80" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E80" s="99"/>
+    <row r="80" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E80" s="88"/>
       <c r="F80" s="4" t="s">
         <v>230</v>
       </c>
@@ -5108,8 +5111,8 @@
         <v>248</v>
       </c>
     </row>
-    <row r="81" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E81" s="99"/>
+    <row r="81" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E81" s="88"/>
       <c r="F81" s="12" t="s">
         <v>231</v>
       </c>
@@ -5138,8 +5141,8 @@
         <v>248</v>
       </c>
     </row>
-    <row r="82" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E82" s="99"/>
+    <row r="82" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E82" s="88"/>
       <c r="F82" s="10" t="s">
         <v>233</v>
       </c>
@@ -5168,8 +5171,8 @@
         <v>248</v>
       </c>
     </row>
-    <row r="85" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E85" s="99" t="s">
+    <row r="85" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E85" s="88" t="s">
         <v>19</v>
       </c>
       <c r="F85" t="s">
@@ -5182,8 +5185,8 @@
         <v>95</v>
       </c>
     </row>
-    <row r="86" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E86" s="99"/>
+    <row r="86" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E86" s="88"/>
       <c r="F86" t="s">
         <v>85</v>
       </c>
@@ -5194,8 +5197,8 @@
         <v>97</v>
       </c>
     </row>
-    <row r="87" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E87" s="99"/>
+    <row r="87" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E87" s="88"/>
       <c r="F87" t="s">
         <v>84</v>
       </c>
@@ -5206,8 +5209,8 @@
         <v>98</v>
       </c>
     </row>
-    <row r="88" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E88" s="99"/>
+    <row r="88" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E88" s="88"/>
       <c r="F88" t="s">
         <v>83</v>
       </c>
@@ -5218,8 +5221,8 @@
         <v>99</v>
       </c>
     </row>
-    <row r="89" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E89" s="99"/>
+    <row r="89" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E89" s="88"/>
       <c r="F89" t="s">
         <v>45</v>
       </c>
@@ -5230,8 +5233,8 @@
         <v>99.5</v>
       </c>
     </row>
-    <row r="90" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E90" s="99"/>
+    <row r="90" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E90" s="88"/>
       <c r="F90" t="s">
         <v>40</v>
       </c>
@@ -5242,8 +5245,8 @@
         <v>99.6</v>
       </c>
     </row>
-    <row r="91" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E91" s="99"/>
+    <row r="91" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E91" s="88"/>
       <c r="F91" t="s">
         <v>44</v>
       </c>
@@ -5254,8 +5257,8 @@
         <v>99.7</v>
       </c>
     </row>
-    <row r="92" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E92" s="99"/>
+    <row r="92" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E92" s="88"/>
       <c r="F92" t="s">
         <v>39</v>
       </c>
@@ -5266,8 +5269,8 @@
         <v>99.8</v>
       </c>
     </row>
-    <row r="93" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E93" s="99"/>
+    <row r="93" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E93" s="88"/>
       <c r="F93" t="s">
         <v>43</v>
       </c>
@@ -5278,8 +5281,8 @@
         <v>99.9</v>
       </c>
     </row>
-    <row r="94" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E94" s="99"/>
+    <row r="94" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E94" s="88"/>
       <c r="F94" t="s">
         <v>42</v>
       </c>
@@ -5290,8 +5293,8 @@
         <v>99.95</v>
       </c>
     </row>
-    <row r="95" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E95" s="99"/>
+    <row r="95" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E95" s="88"/>
       <c r="F95" t="s">
         <v>41</v>
       </c>
@@ -5302,8 +5305,8 @@
         <v>99.96</v>
       </c>
     </row>
-    <row r="96" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E96" s="99"/>
+    <row r="96" spans="5:13" x14ac:dyDescent="0.3">
+      <c r="E96" s="88"/>
       <c r="F96" t="s">
         <v>38</v>
       </c>
@@ -5314,8 +5317,8 @@
         <v>99.97</v>
       </c>
     </row>
-    <row r="97" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E97" s="99"/>
+    <row r="97" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E97" s="88"/>
       <c r="F97" t="s">
         <v>37</v>
       </c>
@@ -5326,8 +5329,8 @@
         <v>99.98</v>
       </c>
     </row>
-    <row r="98" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E98" s="99"/>
+    <row r="98" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E98" s="88"/>
       <c r="F98" t="s">
         <v>36</v>
       </c>
@@ -5338,8 +5341,8 @@
         <v>99.99</v>
       </c>
     </row>
-    <row r="99" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E99" s="99"/>
+    <row r="99" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E99" s="88"/>
       <c r="F99" t="s">
         <v>35</v>
       </c>
@@ -5350,8 +5353,8 @@
         <v>99.995000000000005</v>
       </c>
     </row>
-    <row r="100" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E100" s="99"/>
+    <row r="100" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E100" s="88"/>
       <c r="F100" t="s">
         <v>34</v>
       </c>
@@ -5362,8 +5365,8 @@
         <v>99.995999999999995</v>
       </c>
     </row>
-    <row r="101" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E101" s="99"/>
+    <row r="101" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E101" s="88"/>
       <c r="F101" t="s">
         <v>33</v>
       </c>
@@ -5374,8 +5377,8 @@
         <v>99.997</v>
       </c>
     </row>
-    <row r="102" spans="5:9" x14ac:dyDescent="0.25">
-      <c r="E102" s="99"/>
+    <row r="102" spans="5:9" x14ac:dyDescent="0.3">
+      <c r="E102" s="88"/>
       <c r="F102" t="s">
         <v>32</v>
       </c>
@@ -5386,38 +5389,40 @@
         <v>99.998000000000005</v>
       </c>
     </row>
-    <row r="103" spans="5:9" x14ac:dyDescent="0.25">
+    <row r="103" spans="5:9" x14ac:dyDescent="0.3">
       <c r="I103">
         <v>99.998999999999995</v>
       </c>
     </row>
-    <row r="104" spans="5:9" x14ac:dyDescent="0.25">
+    <row r="104" spans="5:9" x14ac:dyDescent="0.3">
       <c r="I104">
         <v>99.999499999999998</v>
       </c>
     </row>
-    <row r="105" spans="5:9" x14ac:dyDescent="0.25">
+    <row r="105" spans="5:9" x14ac:dyDescent="0.3">
       <c r="I105">
         <v>99.999600000000001</v>
       </c>
     </row>
-    <row r="106" spans="5:9" x14ac:dyDescent="0.25">
+    <row r="106" spans="5:9" x14ac:dyDescent="0.3">
       <c r="I106">
         <v>99.999700000000004</v>
       </c>
     </row>
-    <row r="107" spans="5:9" x14ac:dyDescent="0.25">
+    <row r="107" spans="5:9" x14ac:dyDescent="0.3">
       <c r="I107">
         <v>99.999799999999993</v>
       </c>
     </row>
-    <row r="108" spans="5:9" x14ac:dyDescent="0.25">
+    <row r="108" spans="5:9" x14ac:dyDescent="0.3">
       <c r="I108">
         <v>99.999899999999997</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="E50:E64"/>
     <mergeCell ref="E66:E82"/>
     <mergeCell ref="E85:E102"/>
     <mergeCell ref="A40:A41"/>
@@ -5434,8 +5439,6 @@
     <mergeCell ref="E4:G4"/>
     <mergeCell ref="A7:A11"/>
     <mergeCell ref="A13:A37"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="E50:E64"/>
   </mergeCells>
   <conditionalFormatting sqref="D29">
     <cfRule type="expression" dxfId="12" priority="28">
@@ -5473,25 +5476,25 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="7">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D10">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D10" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"SHE, Kurary"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"1,2,3,4,5,6,7,8,9,10"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D11" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"Max 0% more than required, Max 5% more than required, Max 10% more than required, Max 15% more than required, Max 20% more than required, Full Capacity"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Havayar, Oxymat"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D6" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Havayar"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D29">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D29" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>INDIRECT(CONCATENATE($D$5,".N2.Generator.Models"))</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>$I$85:$I$108</formula1>
     </dataValidation>
   </dataValidations>
@@ -5507,223 +5510,223 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:U48"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" style="54" bestFit="1" customWidth="1"/>
-    <col min="2" max="21" width="6.7109375" style="54" customWidth="1"/>
-    <col min="22" max="22" width="9.140625" style="54" customWidth="1"/>
-    <col min="23" max="16384" width="9.140625" style="54"/>
+    <col min="2" max="21" width="6.6640625" style="54" customWidth="1"/>
+    <col min="22" max="22" width="9.109375" style="54" customWidth="1"/>
+    <col min="23" max="16384" width="9.109375" style="54"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="195"/>
-      <c r="B1" s="196"/>
-      <c r="C1" s="196"/>
-      <c r="D1" s="196"/>
-      <c r="E1" s="196"/>
-      <c r="F1" s="197"/>
-      <c r="G1" s="204" t="str">
+    <row r="1" spans="1:21" ht="35.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="100"/>
+      <c r="B1" s="101"/>
+      <c r="C1" s="101"/>
+      <c r="D1" s="101"/>
+      <c r="E1" s="101"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="109" t="str">
         <f>'[1]Page1-2'!G1:O3</f>
         <v>Title: Data Sheet for HN-700 PSA Nitrogen Generator</v>
       </c>
-      <c r="H1" s="205"/>
-      <c r="I1" s="205"/>
-      <c r="J1" s="205"/>
-      <c r="K1" s="205"/>
-      <c r="L1" s="205"/>
-      <c r="M1" s="205"/>
-      <c r="N1" s="205"/>
-      <c r="O1" s="206"/>
-      <c r="P1" s="213" t="str">
+      <c r="H1" s="110"/>
+      <c r="I1" s="110"/>
+      <c r="J1" s="110"/>
+      <c r="K1" s="110"/>
+      <c r="L1" s="110"/>
+      <c r="M1" s="110"/>
+      <c r="N1" s="110"/>
+      <c r="O1" s="111"/>
+      <c r="P1" s="118" t="str">
         <f>'[1]Page1-2'!P1:U1</f>
         <v>Document Number: HY-ME-DS-N2-0014</v>
       </c>
-      <c r="Q1" s="214"/>
-      <c r="R1" s="214"/>
-      <c r="S1" s="214"/>
-      <c r="T1" s="214"/>
-      <c r="U1" s="215"/>
-    </row>
-    <row r="2" spans="1:21" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="198"/>
-      <c r="B2" s="199"/>
-      <c r="C2" s="199"/>
-      <c r="D2" s="199"/>
-      <c r="E2" s="199"/>
-      <c r="F2" s="200"/>
-      <c r="G2" s="207"/>
-      <c r="H2" s="208"/>
-      <c r="I2" s="208"/>
-      <c r="J2" s="208"/>
-      <c r="K2" s="208"/>
-      <c r="L2" s="208"/>
-      <c r="M2" s="208"/>
-      <c r="N2" s="208"/>
-      <c r="O2" s="209"/>
-      <c r="P2" s="216" t="str">
+      <c r="Q1" s="119"/>
+      <c r="R1" s="119"/>
+      <c r="S1" s="119"/>
+      <c r="T1" s="119"/>
+      <c r="U1" s="120"/>
+    </row>
+    <row r="2" spans="1:21" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="103"/>
+      <c r="B2" s="104"/>
+      <c r="C2" s="104"/>
+      <c r="D2" s="104"/>
+      <c r="E2" s="104"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="112"/>
+      <c r="H2" s="113"/>
+      <c r="I2" s="113"/>
+      <c r="J2" s="113"/>
+      <c r="K2" s="113"/>
+      <c r="L2" s="113"/>
+      <c r="M2" s="113"/>
+      <c r="N2" s="113"/>
+      <c r="O2" s="114"/>
+      <c r="P2" s="121" t="str">
         <f>'[1]Page1-2'!P2:U2</f>
         <v>Rev: 00</v>
       </c>
-      <c r="Q2" s="217"/>
-      <c r="R2" s="217"/>
-      <c r="S2" s="217"/>
-      <c r="T2" s="217"/>
-      <c r="U2" s="218"/>
-    </row>
-    <row r="3" spans="1:21" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="201"/>
-      <c r="B3" s="202"/>
-      <c r="C3" s="202"/>
-      <c r="D3" s="202"/>
-      <c r="E3" s="202"/>
-      <c r="F3" s="203"/>
-      <c r="G3" s="210"/>
-      <c r="H3" s="211"/>
-      <c r="I3" s="211"/>
-      <c r="J3" s="211"/>
-      <c r="K3" s="211"/>
-      <c r="L3" s="211"/>
-      <c r="M3" s="211"/>
-      <c r="N3" s="211"/>
-      <c r="O3" s="212"/>
-      <c r="P3" s="219" t="s">
+      <c r="Q2" s="122"/>
+      <c r="R2" s="122"/>
+      <c r="S2" s="122"/>
+      <c r="T2" s="122"/>
+      <c r="U2" s="123"/>
+    </row>
+    <row r="3" spans="1:21" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="106"/>
+      <c r="B3" s="107"/>
+      <c r="C3" s="107"/>
+      <c r="D3" s="107"/>
+      <c r="E3" s="107"/>
+      <c r="F3" s="108"/>
+      <c r="G3" s="115"/>
+      <c r="H3" s="116"/>
+      <c r="I3" s="116"/>
+      <c r="J3" s="116"/>
+      <c r="K3" s="116"/>
+      <c r="L3" s="116"/>
+      <c r="M3" s="116"/>
+      <c r="N3" s="116"/>
+      <c r="O3" s="117"/>
+      <c r="P3" s="124" t="s">
         <v>103</v>
       </c>
-      <c r="Q3" s="220"/>
-      <c r="R3" s="220"/>
-      <c r="S3" s="220"/>
-      <c r="T3" s="220"/>
-      <c r="U3" s="221"/>
-    </row>
-    <row r="4" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="Q3" s="125"/>
+      <c r="R3" s="125"/>
+      <c r="S3" s="125"/>
+      <c r="T3" s="125"/>
+      <c r="U3" s="126"/>
+    </row>
+    <row r="4" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="55">
         <v>1</v>
       </c>
-      <c r="B4" s="114" t="s">
+      <c r="B4" s="127" t="s">
         <v>104</v>
       </c>
-      <c r="C4" s="115"/>
-      <c r="D4" s="115"/>
-      <c r="E4" s="115"/>
-      <c r="F4" s="115"/>
-      <c r="G4" s="115"/>
-      <c r="H4" s="115"/>
-      <c r="I4" s="115"/>
-      <c r="J4" s="115"/>
-      <c r="K4" s="115"/>
-      <c r="L4" s="115"/>
-      <c r="M4" s="115"/>
-      <c r="N4" s="115"/>
-      <c r="O4" s="115"/>
-      <c r="P4" s="115"/>
-      <c r="Q4" s="115"/>
-      <c r="R4" s="115"/>
-      <c r="S4" s="115"/>
-      <c r="T4" s="115"/>
-      <c r="U4" s="116"/>
-    </row>
-    <row r="5" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C4" s="128"/>
+      <c r="D4" s="128"/>
+      <c r="E4" s="128"/>
+      <c r="F4" s="128"/>
+      <c r="G4" s="128"/>
+      <c r="H4" s="128"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="128"/>
+      <c r="K4" s="128"/>
+      <c r="L4" s="128"/>
+      <c r="M4" s="128"/>
+      <c r="N4" s="128"/>
+      <c r="O4" s="128"/>
+      <c r="P4" s="128"/>
+      <c r="Q4" s="128"/>
+      <c r="R4" s="128"/>
+      <c r="S4" s="128"/>
+      <c r="T4" s="128"/>
+      <c r="U4" s="129"/>
+    </row>
+    <row r="5" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="49">
         <f t="shared" ref="A5:A47" si="0">A4+1</f>
         <v>2</v>
       </c>
-      <c r="B5" s="222" t="s">
+      <c r="B5" s="130" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="223"/>
-      <c r="D5" s="224" t="str">
+      <c r="C5" s="131"/>
+      <c r="D5" s="132" t="str">
         <f>'Equipment Selection'!D29</f>
         <v>N-40x1</v>
       </c>
-      <c r="E5" s="224"/>
-      <c r="F5" s="224"/>
-      <c r="G5" s="225" t="s">
+      <c r="E5" s="132"/>
+      <c r="F5" s="132"/>
+      <c r="G5" s="133" t="s">
         <v>105</v>
       </c>
-      <c r="H5" s="226"/>
-      <c r="I5" s="224" t="s">
+      <c r="H5" s="134"/>
+      <c r="I5" s="132" t="s">
         <v>106</v>
       </c>
-      <c r="J5" s="224"/>
-      <c r="K5" s="224"/>
-      <c r="L5" s="224"/>
-      <c r="M5" s="227" t="s">
+      <c r="J5" s="132"/>
+      <c r="K5" s="132"/>
+      <c r="L5" s="132"/>
+      <c r="M5" s="135" t="s">
         <v>246</v>
       </c>
-      <c r="N5" s="223"/>
-      <c r="O5" s="223"/>
-      <c r="P5" s="224" t="s">
+      <c r="N5" s="131"/>
+      <c r="O5" s="131"/>
+      <c r="P5" s="132" t="s">
         <v>107</v>
       </c>
-      <c r="Q5" s="224"/>
-      <c r="R5" s="224"/>
-      <c r="S5" s="224"/>
-      <c r="T5" s="224"/>
-      <c r="U5" s="228"/>
-    </row>
-    <row r="6" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="Q5" s="132"/>
+      <c r="R5" s="132"/>
+      <c r="S5" s="132"/>
+      <c r="T5" s="132"/>
+      <c r="U5" s="136"/>
+    </row>
+    <row r="6" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="49">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="B6" s="222" t="s">
+      <c r="B6" s="130" t="s">
         <v>247</v>
       </c>
-      <c r="C6" s="223"/>
-      <c r="D6" s="224">
+      <c r="C6" s="131"/>
+      <c r="D6" s="132">
         <f>'Equipment Selection'!D9</f>
         <v>1</v>
       </c>
-      <c r="E6" s="224"/>
-      <c r="F6" s="224"/>
-      <c r="G6" s="225" t="s">
+      <c r="E6" s="132"/>
+      <c r="F6" s="132"/>
+      <c r="G6" s="133" t="s">
         <v>108</v>
       </c>
-      <c r="H6" s="226"/>
-      <c r="I6" s="224" t="s">
+      <c r="H6" s="134"/>
+      <c r="I6" s="132" t="s">
         <v>109</v>
       </c>
-      <c r="J6" s="224"/>
-      <c r="K6" s="224"/>
-      <c r="L6" s="224"/>
-      <c r="M6" s="227" t="s">
+      <c r="J6" s="132"/>
+      <c r="K6" s="132"/>
+      <c r="L6" s="132"/>
+      <c r="M6" s="135" t="s">
         <v>110</v>
       </c>
-      <c r="N6" s="223"/>
-      <c r="O6" s="223"/>
-      <c r="P6" s="224" t="s">
+      <c r="N6" s="131"/>
+      <c r="O6" s="131"/>
+      <c r="P6" s="132" t="s">
         <v>111</v>
       </c>
-      <c r="Q6" s="224"/>
-      <c r="R6" s="224"/>
-      <c r="S6" s="224"/>
-      <c r="T6" s="224"/>
-      <c r="U6" s="228"/>
-    </row>
-    <row r="7" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q6" s="132"/>
+      <c r="R6" s="132"/>
+      <c r="S6" s="132"/>
+      <c r="T6" s="132"/>
+      <c r="U6" s="136"/>
+    </row>
+    <row r="7" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="49">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="B7" s="169" t="s">
+      <c r="B7" s="137" t="s">
         <v>112</v>
       </c>
-      <c r="C7" s="170"/>
-      <c r="D7" s="170"/>
-      <c r="E7" s="170"/>
-      <c r="F7" s="171"/>
-      <c r="G7" s="183" t="str">
+      <c r="C7" s="138"/>
+      <c r="D7" s="138"/>
+      <c r="E7" s="138"/>
+      <c r="F7" s="139"/>
+      <c r="G7" s="151" t="str">
         <f>CONCATENATE('Equipment Selection'!D8,"%")</f>
         <v>99%</v>
       </c>
-      <c r="H7" s="184"/>
-      <c r="I7" s="184"/>
-      <c r="J7" s="185"/>
+      <c r="H7" s="152"/>
+      <c r="I7" s="152"/>
+      <c r="J7" s="153"/>
       <c r="K7" s="78"/>
       <c r="L7" s="77"/>
       <c r="M7" s="78"/>
@@ -5736,25 +5739,25 @@
       <c r="T7" s="58"/>
       <c r="U7" s="59"/>
     </row>
-    <row r="8" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="49">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B8" s="172" t="s">
+      <c r="B8" s="140" t="s">
         <v>113</v>
       </c>
-      <c r="C8" s="173"/>
-      <c r="D8" s="173"/>
-      <c r="E8" s="173"/>
-      <c r="F8" s="173"/>
-      <c r="G8" s="186" t="str">
+      <c r="C8" s="141"/>
+      <c r="D8" s="141"/>
+      <c r="E8" s="141"/>
+      <c r="F8" s="141"/>
+      <c r="G8" s="154" t="str">
         <f>IF('Equipment Selection'!D8&lt;=99.9,CONCATENATE(100-'Equipment Selection'!D8,"%"),CONCATENATE(1000000-10000*'Equipment Selection'!D8,"ppm"))</f>
         <v>1%</v>
       </c>
-      <c r="H8" s="187"/>
-      <c r="I8" s="187"/>
-      <c r="J8" s="188"/>
+      <c r="H8" s="155"/>
+      <c r="I8" s="155"/>
+      <c r="J8" s="156"/>
       <c r="K8" s="86"/>
       <c r="L8" s="79"/>
       <c r="M8" s="79"/>
@@ -5767,25 +5770,25 @@
       <c r="T8" s="61"/>
       <c r="U8" s="62"/>
     </row>
-    <row r="9" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="49">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="B9" s="172" t="s">
+      <c r="B9" s="140" t="s">
         <v>114</v>
       </c>
-      <c r="C9" s="173"/>
-      <c r="D9" s="173"/>
-      <c r="E9" s="173"/>
-      <c r="F9" s="173"/>
-      <c r="G9" s="186" t="str">
+      <c r="C9" s="141"/>
+      <c r="D9" s="141"/>
+      <c r="E9" s="141"/>
+      <c r="F9" s="141"/>
+      <c r="G9" s="154" t="str">
         <f ca="1">CONCATENATE(D6,"x",ROUNDUP('Equipment Selection'!D36/Datasheet!D6/0.92,2))</f>
         <v>1x3.75</v>
       </c>
-      <c r="H9" s="187"/>
-      <c r="I9" s="187"/>
-      <c r="J9" s="188"/>
+      <c r="H9" s="155"/>
+      <c r="I9" s="155"/>
+      <c r="J9" s="156"/>
       <c r="K9" s="81"/>
       <c r="L9" s="80"/>
       <c r="M9" s="81"/>
@@ -5798,25 +5801,25 @@
       <c r="T9" s="63"/>
       <c r="U9" s="64"/>
     </row>
-    <row r="10" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="49">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="B10" s="172" t="s">
+      <c r="B10" s="140" t="s">
         <v>261</v>
       </c>
-      <c r="C10" s="173"/>
-      <c r="D10" s="173"/>
-      <c r="E10" s="173"/>
-      <c r="F10" s="173"/>
-      <c r="G10" s="186" t="str">
+      <c r="C10" s="141"/>
+      <c r="D10" s="141"/>
+      <c r="E10" s="141"/>
+      <c r="F10" s="141"/>
+      <c r="G10" s="154" t="str">
         <f ca="1">CONCATENATE(D6,"x",ROUNDUP('Equipment Selection'!D37/Datasheet!D6/60,2))</f>
         <v>1x0.2</v>
       </c>
-      <c r="H10" s="187"/>
-      <c r="I10" s="187"/>
-      <c r="J10" s="188"/>
+      <c r="H10" s="155"/>
+      <c r="I10" s="155"/>
+      <c r="J10" s="156"/>
       <c r="K10" s="83"/>
       <c r="L10" s="82"/>
       <c r="M10" s="83"/>
@@ -5829,25 +5832,25 @@
       <c r="T10" s="65"/>
       <c r="U10" s="66"/>
     </row>
-    <row r="11" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="49">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="B11" s="172" t="s">
+      <c r="B11" s="140" t="s">
         <v>115</v>
       </c>
-      <c r="C11" s="173"/>
-      <c r="D11" s="173"/>
-      <c r="E11" s="173"/>
-      <c r="F11" s="173"/>
-      <c r="G11" s="189">
+      <c r="C11" s="141"/>
+      <c r="D11" s="141"/>
+      <c r="E11" s="141"/>
+      <c r="F11" s="141"/>
+      <c r="G11" s="157">
         <f ca="1">ROUNDUP('Equipment Selection'!D40,-2)</f>
         <v>100</v>
       </c>
-      <c r="H11" s="190"/>
-      <c r="I11" s="190"/>
-      <c r="J11" s="191"/>
+      <c r="H11" s="158"/>
+      <c r="I11" s="158"/>
+      <c r="J11" s="159"/>
       <c r="K11" s="85"/>
       <c r="L11" s="84"/>
       <c r="M11" s="85"/>
@@ -5860,25 +5863,25 @@
       <c r="T11" s="67"/>
       <c r="U11" s="68"/>
     </row>
-    <row r="12" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="49">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="B12" s="174" t="s">
+      <c r="B12" s="142" t="s">
         <v>116</v>
       </c>
-      <c r="C12" s="175"/>
-      <c r="D12" s="175"/>
-      <c r="E12" s="175"/>
-      <c r="F12" s="175"/>
-      <c r="G12" s="192">
+      <c r="C12" s="143"/>
+      <c r="D12" s="143"/>
+      <c r="E12" s="143"/>
+      <c r="F12" s="143"/>
+      <c r="G12" s="160">
         <f ca="1">ROUNDUP('Equipment Selection'!D38,-2)</f>
         <v>100</v>
       </c>
-      <c r="H12" s="193"/>
-      <c r="I12" s="193"/>
-      <c r="J12" s="194"/>
+      <c r="H12" s="161"/>
+      <c r="I12" s="161"/>
+      <c r="J12" s="162"/>
       <c r="K12" s="85"/>
       <c r="L12" s="84"/>
       <c r="M12" s="85"/>
@@ -5891,770 +5894,770 @@
       <c r="T12" s="67"/>
       <c r="U12" s="68"/>
     </row>
-    <row r="13" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="49">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="B13" s="176" t="s">
+      <c r="B13" s="144" t="s">
         <v>117</v>
       </c>
-      <c r="C13" s="177"/>
-      <c r="D13" s="178"/>
-      <c r="E13" s="179">
+      <c r="C13" s="145"/>
+      <c r="D13" s="146"/>
+      <c r="E13" s="147">
         <v>2000</v>
       </c>
-      <c r="F13" s="180"/>
-      <c r="G13" s="180"/>
-      <c r="H13" s="181" t="s">
+      <c r="F13" s="148"/>
+      <c r="G13" s="148"/>
+      <c r="H13" s="149" t="s">
         <v>118</v>
       </c>
-      <c r="I13" s="181"/>
-      <c r="J13" s="181"/>
-      <c r="K13" s="182"/>
-      <c r="L13" s="157">
+      <c r="I13" s="149"/>
+      <c r="J13" s="149"/>
+      <c r="K13" s="150"/>
+      <c r="L13" s="163">
         <f ca="1">'Equipment Selection'!D34</f>
         <v>15.298090597274824</v>
       </c>
-      <c r="M13" s="158"/>
-      <c r="N13" s="158"/>
-      <c r="O13" s="159"/>
-      <c r="P13" s="160"/>
-      <c r="Q13" s="160"/>
-      <c r="R13" s="160"/>
-      <c r="S13" s="160"/>
-      <c r="T13" s="160"/>
-      <c r="U13" s="161"/>
-    </row>
-    <row r="14" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M13" s="164"/>
+      <c r="N13" s="164"/>
+      <c r="O13" s="165"/>
+      <c r="P13" s="166"/>
+      <c r="Q13" s="166"/>
+      <c r="R13" s="166"/>
+      <c r="S13" s="166"/>
+      <c r="T13" s="166"/>
+      <c r="U13" s="167"/>
+    </row>
+    <row r="14" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="49">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="B14" s="162" t="s">
+      <c r="B14" s="168" t="s">
         <v>227</v>
       </c>
-      <c r="C14" s="163"/>
-      <c r="D14" s="163"/>
-      <c r="E14" s="164"/>
+      <c r="C14" s="169"/>
+      <c r="D14" s="169"/>
+      <c r="E14" s="170"/>
       <c r="F14" s="73">
         <f>'Equipment Selection'!D2</f>
         <v>8.5</v>
       </c>
-      <c r="G14" s="149" t="s">
+      <c r="G14" s="171" t="s">
         <v>119</v>
       </c>
-      <c r="H14" s="149"/>
-      <c r="I14" s="150"/>
-      <c r="J14" s="165">
+      <c r="H14" s="171"/>
+      <c r="I14" s="172"/>
+      <c r="J14" s="173">
         <f>'Equipment Selection'!D12</f>
         <v>7.7</v>
       </c>
-      <c r="K14" s="166"/>
-      <c r="L14" s="149" t="s">
+      <c r="K14" s="174"/>
+      <c r="L14" s="171" t="s">
         <v>120</v>
       </c>
-      <c r="M14" s="149"/>
-      <c r="N14" s="150"/>
-      <c r="O14" s="167" t="str">
+      <c r="M14" s="171"/>
+      <c r="N14" s="172"/>
+      <c r="O14" s="175" t="str">
         <f>CONCATENATE(IF('Equipment Selection'!D8&gt;99.99,"-20","+3")," or less")</f>
         <v>+3 or less</v>
       </c>
-      <c r="P14" s="168"/>
-      <c r="Q14" s="149" t="s">
+      <c r="P14" s="176"/>
+      <c r="Q14" s="171" t="s">
         <v>121</v>
       </c>
-      <c r="R14" s="149"/>
-      <c r="S14" s="149"/>
-      <c r="T14" s="150"/>
+      <c r="R14" s="171"/>
+      <c r="S14" s="171"/>
+      <c r="T14" s="172"/>
       <c r="U14" s="69">
         <f>'Equipment Selection'!D4</f>
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="49">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="B15" s="151" t="s">
+      <c r="B15" s="183" t="s">
         <v>122</v>
       </c>
-      <c r="C15" s="152"/>
-      <c r="D15" s="152"/>
-      <c r="E15" s="152"/>
-      <c r="F15" s="153" t="str">
+      <c r="C15" s="184"/>
+      <c r="D15" s="184"/>
+      <c r="E15" s="184"/>
+      <c r="F15" s="185" t="str">
         <f ca="1">INDEX(INDIRECT(CONCATENATE('Equipment Selection'!D5,".N2.Generator.Dimensions")),MATCH('Equipment Selection'!D29,INDIRECT(CONCATENATE('Equipment Selection'!D5,".N2.Generator.Models")),0))</f>
         <v>50x60x150</v>
       </c>
-      <c r="G15" s="154"/>
-      <c r="H15" s="152" t="s">
+      <c r="G15" s="186"/>
+      <c r="H15" s="184" t="s">
         <v>123</v>
       </c>
-      <c r="I15" s="152"/>
-      <c r="J15" s="152"/>
-      <c r="K15" s="152"/>
-      <c r="L15" s="152"/>
-      <c r="M15" s="153" t="str">
+      <c r="I15" s="184"/>
+      <c r="J15" s="184"/>
+      <c r="K15" s="184"/>
+      <c r="L15" s="184"/>
+      <c r="M15" s="185" t="str">
         <f ca="1">CONCATENATE(LEFT(F15,SEARCH("x",F15)-1)+20,"x",MID(F15,SEARCH("x",F15)+1,SEARCH("x",F15,5)-SEARCH("x",F15)-1)+20,"x",RIGHT(F15,3)+25)</f>
         <v>70x80x175</v>
       </c>
-      <c r="N15" s="154"/>
-      <c r="O15" s="112" t="s">
+      <c r="N15" s="186"/>
+      <c r="O15" s="187" t="s">
         <v>124</v>
       </c>
-      <c r="P15" s="112"/>
-      <c r="Q15" s="112"/>
-      <c r="R15" s="112"/>
-      <c r="S15" s="112"/>
-      <c r="T15" s="155" t="str">
+      <c r="P15" s="187"/>
+      <c r="Q15" s="187"/>
+      <c r="R15" s="187"/>
+      <c r="S15" s="187"/>
+      <c r="T15" s="188" t="str">
         <f ca="1">CONCATENATE(LEFT(F15,SEARCH("x",F15)-1)+20,"x",MID(F15,SEARCH("x",F15)+1,SEARCH("x",F15,5)-SEARCH("x",F15)-1)+70,"x",RIGHT(F15,3)+20)</f>
         <v>70x130x170</v>
       </c>
-      <c r="U15" s="156"/>
-    </row>
-    <row r="16" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="U15" s="189"/>
+    </row>
+    <row r="16" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="49">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="B16" s="114" t="s">
+      <c r="B16" s="127" t="s">
         <v>125</v>
       </c>
-      <c r="C16" s="115"/>
-      <c r="D16" s="115"/>
-      <c r="E16" s="115"/>
-      <c r="F16" s="115"/>
-      <c r="G16" s="115"/>
-      <c r="H16" s="115"/>
-      <c r="I16" s="115"/>
-      <c r="J16" s="116"/>
-      <c r="K16" s="114" t="s">
+      <c r="C16" s="128"/>
+      <c r="D16" s="128"/>
+      <c r="E16" s="128"/>
+      <c r="F16" s="128"/>
+      <c r="G16" s="128"/>
+      <c r="H16" s="128"/>
+      <c r="I16" s="128"/>
+      <c r="J16" s="129"/>
+      <c r="K16" s="127" t="s">
         <v>126</v>
       </c>
-      <c r="L16" s="115"/>
-      <c r="M16" s="115"/>
-      <c r="N16" s="115"/>
-      <c r="O16" s="115"/>
-      <c r="P16" s="115"/>
-      <c r="Q16" s="115"/>
-      <c r="R16" s="115"/>
-      <c r="S16" s="115"/>
-      <c r="T16" s="115"/>
-      <c r="U16" s="116"/>
-    </row>
-    <row r="17" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L16" s="128"/>
+      <c r="M16" s="128"/>
+      <c r="N16" s="128"/>
+      <c r="O16" s="128"/>
+      <c r="P16" s="128"/>
+      <c r="Q16" s="128"/>
+      <c r="R16" s="128"/>
+      <c r="S16" s="128"/>
+      <c r="T16" s="128"/>
+      <c r="U16" s="129"/>
+    </row>
+    <row r="17" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="49">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="B17" s="136" t="s">
+      <c r="B17" s="177" t="s">
         <v>127</v>
       </c>
-      <c r="C17" s="137"/>
-      <c r="D17" s="137"/>
-      <c r="E17" s="137"/>
-      <c r="F17" s="137"/>
-      <c r="G17" s="137"/>
-      <c r="H17" s="103" t="s">
+      <c r="C17" s="178"/>
+      <c r="D17" s="178"/>
+      <c r="E17" s="178"/>
+      <c r="F17" s="178"/>
+      <c r="G17" s="178"/>
+      <c r="H17" s="179" t="s">
         <v>128</v>
       </c>
-      <c r="I17" s="103"/>
-      <c r="J17" s="104"/>
-      <c r="K17" s="136" t="s">
+      <c r="I17" s="179"/>
+      <c r="J17" s="180"/>
+      <c r="K17" s="177" t="s">
         <v>129</v>
       </c>
-      <c r="L17" s="137"/>
-      <c r="M17" s="147" t="s">
+      <c r="L17" s="178"/>
+      <c r="M17" s="181" t="s">
         <v>130</v>
       </c>
-      <c r="N17" s="147"/>
+      <c r="N17" s="181"/>
       <c r="O17" s="50" t="s">
         <v>131</v>
       </c>
-      <c r="P17" s="147" t="s">
+      <c r="P17" s="181" t="s">
         <v>132</v>
       </c>
-      <c r="Q17" s="147"/>
-      <c r="R17" s="147" t="s">
+      <c r="Q17" s="181"/>
+      <c r="R17" s="181" t="s">
         <v>64</v>
       </c>
-      <c r="S17" s="147"/>
-      <c r="T17" s="147"/>
-      <c r="U17" s="148"/>
-    </row>
-    <row r="18" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S17" s="181"/>
+      <c r="T17" s="181"/>
+      <c r="U17" s="182"/>
+    </row>
+    <row r="18" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="49">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="B18" s="136" t="s">
+      <c r="B18" s="177" t="s">
         <v>133</v>
       </c>
-      <c r="C18" s="137"/>
-      <c r="D18" s="137"/>
-      <c r="E18" s="137"/>
-      <c r="F18" s="137"/>
-      <c r="G18" s="137"/>
-      <c r="H18" s="138" t="s">
+      <c r="C18" s="178"/>
+      <c r="D18" s="178"/>
+      <c r="E18" s="178"/>
+      <c r="F18" s="178"/>
+      <c r="G18" s="178"/>
+      <c r="H18" s="190" t="s">
         <v>134</v>
       </c>
-      <c r="I18" s="138"/>
-      <c r="J18" s="139"/>
-      <c r="K18" s="144" t="s">
+      <c r="I18" s="190"/>
+      <c r="J18" s="191"/>
+      <c r="K18" s="192" t="s">
         <v>135</v>
       </c>
-      <c r="L18" s="145"/>
-      <c r="M18" s="103" t="s">
+      <c r="L18" s="193"/>
+      <c r="M18" s="179" t="s">
         <v>136</v>
       </c>
-      <c r="N18" s="103"/>
+      <c r="N18" s="179"/>
       <c r="O18" s="51" t="s">
         <v>137</v>
       </c>
-      <c r="P18" s="103" t="s">
+      <c r="P18" s="179" t="s">
         <v>138</v>
       </c>
-      <c r="Q18" s="103"/>
-      <c r="R18" s="146" t="s">
+      <c r="Q18" s="179"/>
+      <c r="R18" s="194" t="s">
         <v>4</v>
       </c>
-      <c r="S18" s="103"/>
-      <c r="T18" s="103"/>
-      <c r="U18" s="104"/>
-    </row>
-    <row r="19" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S18" s="179"/>
+      <c r="T18" s="179"/>
+      <c r="U18" s="180"/>
+    </row>
+    <row r="19" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="49">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="B19" s="136" t="s">
+      <c r="B19" s="177" t="s">
         <v>139</v>
       </c>
-      <c r="C19" s="137"/>
-      <c r="D19" s="137"/>
-      <c r="E19" s="137"/>
-      <c r="F19" s="137"/>
-      <c r="G19" s="137"/>
-      <c r="H19" s="138">
+      <c r="C19" s="178"/>
+      <c r="D19" s="178"/>
+      <c r="E19" s="178"/>
+      <c r="F19" s="178"/>
+      <c r="G19" s="178"/>
+      <c r="H19" s="190">
         <v>85</v>
       </c>
-      <c r="I19" s="138"/>
-      <c r="J19" s="139"/>
-      <c r="K19" s="144" t="s">
+      <c r="I19" s="190"/>
+      <c r="J19" s="191"/>
+      <c r="K19" s="192" t="s">
         <v>140</v>
       </c>
-      <c r="L19" s="145"/>
-      <c r="M19" s="103" t="s">
+      <c r="L19" s="193"/>
+      <c r="M19" s="179" t="s">
         <v>136</v>
       </c>
-      <c r="N19" s="103"/>
+      <c r="N19" s="179"/>
       <c r="O19" s="51" t="s">
         <v>137</v>
       </c>
-      <c r="P19" s="103" t="s">
+      <c r="P19" s="179" t="s">
         <v>138</v>
       </c>
-      <c r="Q19" s="103"/>
-      <c r="R19" s="146" t="s">
+      <c r="Q19" s="179"/>
+      <c r="R19" s="194" t="s">
         <v>141</v>
       </c>
-      <c r="S19" s="103"/>
-      <c r="T19" s="103"/>
-      <c r="U19" s="104"/>
-    </row>
-    <row r="20" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S19" s="179"/>
+      <c r="T19" s="179"/>
+      <c r="U19" s="180"/>
+    </row>
+    <row r="20" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="49">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="B20" s="136" t="s">
+      <c r="B20" s="177" t="s">
         <v>142</v>
       </c>
-      <c r="C20" s="137"/>
-      <c r="D20" s="137"/>
-      <c r="E20" s="137"/>
-      <c r="F20" s="137"/>
-      <c r="G20" s="137"/>
-      <c r="H20" s="138">
+      <c r="C20" s="178"/>
+      <c r="D20" s="178"/>
+      <c r="E20" s="178"/>
+      <c r="F20" s="178"/>
+      <c r="G20" s="178"/>
+      <c r="H20" s="190">
         <v>0.5</v>
       </c>
-      <c r="I20" s="138"/>
-      <c r="J20" s="139"/>
-      <c r="K20" s="144" t="s">
+      <c r="I20" s="190"/>
+      <c r="J20" s="191"/>
+      <c r="K20" s="192" t="s">
         <v>143</v>
       </c>
-      <c r="L20" s="145"/>
-      <c r="M20" s="103" t="s">
+      <c r="L20" s="193"/>
+      <c r="M20" s="179" t="s">
         <v>144</v>
       </c>
-      <c r="N20" s="103"/>
+      <c r="N20" s="179"/>
       <c r="O20" s="51" t="s">
         <v>137</v>
       </c>
-      <c r="P20" s="103" t="s">
+      <c r="P20" s="179" t="s">
         <v>138</v>
       </c>
-      <c r="Q20" s="103"/>
-      <c r="R20" s="103" t="s">
+      <c r="Q20" s="179"/>
+      <c r="R20" s="179" t="s">
         <v>145</v>
       </c>
-      <c r="S20" s="103"/>
-      <c r="T20" s="103"/>
-      <c r="U20" s="104"/>
-    </row>
-    <row r="21" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S20" s="179"/>
+      <c r="T20" s="179"/>
+      <c r="U20" s="180"/>
+    </row>
+    <row r="21" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="49">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="B21" s="136" t="s">
+      <c r="B21" s="177" t="s">
         <v>146</v>
       </c>
-      <c r="C21" s="137"/>
-      <c r="D21" s="137"/>
-      <c r="E21" s="137"/>
-      <c r="F21" s="137"/>
-      <c r="G21" s="137"/>
-      <c r="H21" s="138" t="s">
+      <c r="C21" s="178"/>
+      <c r="D21" s="178"/>
+      <c r="E21" s="178"/>
+      <c r="F21" s="178"/>
+      <c r="G21" s="178"/>
+      <c r="H21" s="190" t="s">
         <v>147</v>
       </c>
-      <c r="I21" s="138"/>
-      <c r="J21" s="139"/>
-      <c r="K21" s="144" t="s">
+      <c r="I21" s="190"/>
+      <c r="J21" s="191"/>
+      <c r="K21" s="192" t="s">
         <v>148</v>
       </c>
-      <c r="L21" s="145"/>
-      <c r="M21" s="103" t="s">
+      <c r="L21" s="193"/>
+      <c r="M21" s="179" t="s">
         <v>149</v>
       </c>
-      <c r="N21" s="103"/>
-      <c r="O21" s="103" t="s">
+      <c r="N21" s="179"/>
+      <c r="O21" s="179" t="s">
         <v>150</v>
       </c>
-      <c r="P21" s="103"/>
-      <c r="Q21" s="103"/>
-      <c r="R21" s="103" t="s">
+      <c r="P21" s="179"/>
+      <c r="Q21" s="179"/>
+      <c r="R21" s="179" t="s">
         <v>151</v>
       </c>
-      <c r="S21" s="103"/>
-      <c r="T21" s="103"/>
-      <c r="U21" s="104"/>
-    </row>
-    <row r="22" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="S21" s="179"/>
+      <c r="T21" s="179"/>
+      <c r="U21" s="180"/>
+    </row>
+    <row r="22" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="49">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="B22" s="136" t="s">
+      <c r="B22" s="177" t="s">
         <v>152</v>
       </c>
-      <c r="C22" s="137"/>
-      <c r="D22" s="137"/>
-      <c r="E22" s="137"/>
-      <c r="F22" s="137"/>
-      <c r="G22" s="137"/>
-      <c r="H22" s="138" t="s">
+      <c r="C22" s="178"/>
+      <c r="D22" s="178"/>
+      <c r="E22" s="178"/>
+      <c r="F22" s="178"/>
+      <c r="G22" s="178"/>
+      <c r="H22" s="190" t="s">
         <v>153</v>
       </c>
-      <c r="I22" s="138"/>
-      <c r="J22" s="139"/>
-      <c r="K22" s="114" t="s">
+      <c r="I22" s="190"/>
+      <c r="J22" s="191"/>
+      <c r="K22" s="127" t="s">
         <v>154</v>
       </c>
-      <c r="L22" s="115"/>
-      <c r="M22" s="115"/>
-      <c r="N22" s="115"/>
-      <c r="O22" s="115"/>
-      <c r="P22" s="115"/>
-      <c r="Q22" s="115"/>
-      <c r="R22" s="115"/>
-      <c r="S22" s="115"/>
-      <c r="T22" s="115"/>
-      <c r="U22" s="116"/>
-    </row>
-    <row r="23" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L22" s="128"/>
+      <c r="M22" s="128"/>
+      <c r="N22" s="128"/>
+      <c r="O22" s="128"/>
+      <c r="P22" s="128"/>
+      <c r="Q22" s="128"/>
+      <c r="R22" s="128"/>
+      <c r="S22" s="128"/>
+      <c r="T22" s="128"/>
+      <c r="U22" s="129"/>
+    </row>
+    <row r="23" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="49">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="B23" s="136" t="s">
+      <c r="B23" s="177" t="s">
         <v>155</v>
       </c>
-      <c r="C23" s="137"/>
-      <c r="D23" s="137"/>
-      <c r="E23" s="137"/>
-      <c r="F23" s="137"/>
-      <c r="G23" s="137"/>
-      <c r="H23" s="138" t="s">
+      <c r="C23" s="178"/>
+      <c r="D23" s="178"/>
+      <c r="E23" s="178"/>
+      <c r="F23" s="178"/>
+      <c r="G23" s="178"/>
+      <c r="H23" s="190" t="s">
         <v>156</v>
       </c>
-      <c r="I23" s="138"/>
-      <c r="J23" s="139"/>
-      <c r="K23" s="140" t="s">
+      <c r="I23" s="190"/>
+      <c r="J23" s="191"/>
+      <c r="K23" s="197" t="s">
         <v>157</v>
       </c>
-      <c r="L23" s="141"/>
-      <c r="M23" s="141"/>
-      <c r="N23" s="141"/>
-      <c r="O23" s="142" t="s">
+      <c r="L23" s="198"/>
+      <c r="M23" s="198"/>
+      <c r="N23" s="198"/>
+      <c r="O23" s="199" t="s">
         <v>158</v>
       </c>
-      <c r="P23" s="142"/>
-      <c r="Q23" s="142"/>
-      <c r="R23" s="142"/>
-      <c r="S23" s="142"/>
-      <c r="T23" s="142"/>
-      <c r="U23" s="143"/>
-    </row>
-    <row r="24" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P23" s="199"/>
+      <c r="Q23" s="199"/>
+      <c r="R23" s="199"/>
+      <c r="S23" s="199"/>
+      <c r="T23" s="199"/>
+      <c r="U23" s="200"/>
+    </row>
+    <row r="24" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="49">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="B24" s="136" t="s">
+      <c r="B24" s="177" t="s">
         <v>159</v>
       </c>
-      <c r="C24" s="137"/>
-      <c r="D24" s="137"/>
-      <c r="E24" s="137"/>
-      <c r="F24" s="137"/>
-      <c r="G24" s="137"/>
-      <c r="H24" s="138" t="s">
+      <c r="C24" s="178"/>
+      <c r="D24" s="178"/>
+      <c r="E24" s="178"/>
+      <c r="F24" s="178"/>
+      <c r="G24" s="178"/>
+      <c r="H24" s="190" t="s">
         <v>160</v>
       </c>
-      <c r="I24" s="138"/>
-      <c r="J24" s="139"/>
-      <c r="K24" s="136" t="s">
+      <c r="I24" s="190"/>
+      <c r="J24" s="191"/>
+      <c r="K24" s="177" t="s">
         <v>161</v>
       </c>
-      <c r="L24" s="137"/>
-      <c r="M24" s="137"/>
-      <c r="N24" s="137"/>
-      <c r="O24" s="138" t="s">
+      <c r="L24" s="178"/>
+      <c r="M24" s="178"/>
+      <c r="N24" s="178"/>
+      <c r="O24" s="190" t="s">
         <v>162</v>
       </c>
-      <c r="P24" s="138"/>
-      <c r="Q24" s="138"/>
-      <c r="R24" s="138"/>
-      <c r="S24" s="138"/>
-      <c r="T24" s="138"/>
-      <c r="U24" s="139"/>
-    </row>
-    <row r="25" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="P24" s="190"/>
+      <c r="Q24" s="190"/>
+      <c r="R24" s="190"/>
+      <c r="S24" s="190"/>
+      <c r="T24" s="190"/>
+      <c r="U24" s="191"/>
+    </row>
+    <row r="25" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="49">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="B25" s="136" t="s">
+      <c r="B25" s="177" t="s">
         <v>163</v>
       </c>
-      <c r="C25" s="137"/>
-      <c r="D25" s="137"/>
-      <c r="E25" s="137"/>
-      <c r="F25" s="137"/>
-      <c r="G25" s="137"/>
-      <c r="H25" s="138" t="s">
+      <c r="C25" s="178"/>
+      <c r="D25" s="178"/>
+      <c r="E25" s="178"/>
+      <c r="F25" s="178"/>
+      <c r="G25" s="178"/>
+      <c r="H25" s="190" t="s">
         <v>164</v>
       </c>
-      <c r="I25" s="138"/>
-      <c r="J25" s="139"/>
-      <c r="K25" s="130" t="s">
+      <c r="I25" s="190"/>
+      <c r="J25" s="191"/>
+      <c r="K25" s="195" t="s">
         <v>165</v>
       </c>
-      <c r="L25" s="131"/>
-      <c r="M25" s="131"/>
-      <c r="N25" s="131"/>
-      <c r="O25" s="103" t="s">
+      <c r="L25" s="196"/>
+      <c r="M25" s="196"/>
+      <c r="N25" s="196"/>
+      <c r="O25" s="179" t="s">
         <v>166</v>
       </c>
-      <c r="P25" s="103"/>
-      <c r="Q25" s="103"/>
-      <c r="R25" s="103"/>
-      <c r="S25" s="103"/>
-      <c r="T25" s="103"/>
-      <c r="U25" s="104"/>
-    </row>
-    <row r="26" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="P25" s="179"/>
+      <c r="Q25" s="179"/>
+      <c r="R25" s="179"/>
+      <c r="S25" s="179"/>
+      <c r="T25" s="179"/>
+      <c r="U25" s="180"/>
+    </row>
+    <row r="26" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="49">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="B26" s="114" t="s">
+      <c r="B26" s="127" t="s">
         <v>167</v>
       </c>
-      <c r="C26" s="115"/>
-      <c r="D26" s="115"/>
-      <c r="E26" s="115"/>
-      <c r="F26" s="115"/>
-      <c r="G26" s="115"/>
-      <c r="H26" s="115"/>
-      <c r="I26" s="115"/>
-      <c r="J26" s="116"/>
-      <c r="K26" s="130" t="s">
+      <c r="C26" s="128"/>
+      <c r="D26" s="128"/>
+      <c r="E26" s="128"/>
+      <c r="F26" s="128"/>
+      <c r="G26" s="128"/>
+      <c r="H26" s="128"/>
+      <c r="I26" s="128"/>
+      <c r="J26" s="129"/>
+      <c r="K26" s="195" t="s">
         <v>168</v>
       </c>
-      <c r="L26" s="131"/>
-      <c r="M26" s="131"/>
-      <c r="N26" s="131"/>
-      <c r="O26" s="103" t="s">
+      <c r="L26" s="196"/>
+      <c r="M26" s="196"/>
+      <c r="N26" s="196"/>
+      <c r="O26" s="179" t="s">
         <v>169</v>
       </c>
-      <c r="P26" s="103"/>
-      <c r="Q26" s="103"/>
-      <c r="R26" s="103"/>
-      <c r="S26" s="103"/>
-      <c r="T26" s="103"/>
-      <c r="U26" s="104"/>
-    </row>
-    <row r="27" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P26" s="179"/>
+      <c r="Q26" s="179"/>
+      <c r="R26" s="179"/>
+      <c r="S26" s="179"/>
+      <c r="T26" s="179"/>
+      <c r="U26" s="180"/>
+    </row>
+    <row r="27" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="49">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="B27" s="101" t="s">
+      <c r="B27" s="201" t="s">
         <v>170</v>
       </c>
-      <c r="C27" s="102"/>
-      <c r="D27" s="102"/>
-      <c r="E27" s="102"/>
-      <c r="F27" s="103" t="s">
+      <c r="C27" s="202"/>
+      <c r="D27" s="202"/>
+      <c r="E27" s="202"/>
+      <c r="F27" s="179" t="s">
         <v>171</v>
       </c>
-      <c r="G27" s="103"/>
-      <c r="H27" s="103"/>
-      <c r="I27" s="103"/>
-      <c r="J27" s="104"/>
-      <c r="K27" s="130" t="s">
+      <c r="G27" s="179"/>
+      <c r="H27" s="179"/>
+      <c r="I27" s="179"/>
+      <c r="J27" s="180"/>
+      <c r="K27" s="195" t="s">
         <v>172</v>
       </c>
-      <c r="L27" s="131"/>
-      <c r="M27" s="131"/>
-      <c r="N27" s="131"/>
-      <c r="O27" s="103" t="s">
+      <c r="L27" s="196"/>
+      <c r="M27" s="196"/>
+      <c r="N27" s="196"/>
+      <c r="O27" s="179" t="s">
         <v>173</v>
       </c>
-      <c r="P27" s="103"/>
-      <c r="Q27" s="103"/>
-      <c r="R27" s="103"/>
-      <c r="S27" s="103"/>
-      <c r="T27" s="103"/>
-      <c r="U27" s="104"/>
-    </row>
-    <row r="28" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P27" s="179"/>
+      <c r="Q27" s="179"/>
+      <c r="R27" s="179"/>
+      <c r="S27" s="179"/>
+      <c r="T27" s="179"/>
+      <c r="U27" s="180"/>
+    </row>
+    <row r="28" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="49">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="B28" s="101" t="s">
+      <c r="B28" s="201" t="s">
         <v>174</v>
       </c>
-      <c r="C28" s="102"/>
-      <c r="D28" s="102"/>
-      <c r="E28" s="102"/>
-      <c r="F28" s="103" t="s">
+      <c r="C28" s="202"/>
+      <c r="D28" s="202"/>
+      <c r="E28" s="202"/>
+      <c r="F28" s="179" t="s">
         <v>175</v>
       </c>
-      <c r="G28" s="103"/>
-      <c r="H28" s="103"/>
-      <c r="I28" s="103"/>
-      <c r="J28" s="104"/>
-      <c r="K28" s="130" t="s">
+      <c r="G28" s="179"/>
+      <c r="H28" s="179"/>
+      <c r="I28" s="179"/>
+      <c r="J28" s="180"/>
+      <c r="K28" s="195" t="s">
         <v>176</v>
       </c>
-      <c r="L28" s="131"/>
-      <c r="M28" s="131"/>
-      <c r="N28" s="131"/>
-      <c r="O28" s="103" t="s">
+      <c r="L28" s="196"/>
+      <c r="M28" s="196"/>
+      <c r="N28" s="196"/>
+      <c r="O28" s="179" t="s">
         <v>177</v>
       </c>
-      <c r="P28" s="103"/>
-      <c r="Q28" s="103"/>
-      <c r="R28" s="103"/>
-      <c r="S28" s="103"/>
-      <c r="T28" s="103"/>
-      <c r="U28" s="104"/>
-    </row>
-    <row r="29" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P28" s="179"/>
+      <c r="Q28" s="179"/>
+      <c r="R28" s="179"/>
+      <c r="S28" s="179"/>
+      <c r="T28" s="179"/>
+      <c r="U28" s="180"/>
+    </row>
+    <row r="29" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="49">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="B29" s="101" t="s">
+      <c r="B29" s="201" t="s">
         <v>178</v>
       </c>
-      <c r="C29" s="102"/>
-      <c r="D29" s="102"/>
-      <c r="E29" s="102"/>
-      <c r="F29" s="134" t="s">
+      <c r="C29" s="202"/>
+      <c r="D29" s="202"/>
+      <c r="E29" s="202"/>
+      <c r="F29" s="203" t="s">
         <v>179</v>
       </c>
-      <c r="G29" s="134"/>
-      <c r="H29" s="134"/>
-      <c r="I29" s="134"/>
-      <c r="J29" s="135"/>
-      <c r="K29" s="130" t="s">
+      <c r="G29" s="203"/>
+      <c r="H29" s="203"/>
+      <c r="I29" s="203"/>
+      <c r="J29" s="204"/>
+      <c r="K29" s="195" t="s">
         <v>180</v>
       </c>
-      <c r="L29" s="131"/>
-      <c r="M29" s="131"/>
-      <c r="N29" s="131"/>
-      <c r="O29" s="103" t="s">
+      <c r="L29" s="196"/>
+      <c r="M29" s="196"/>
+      <c r="N29" s="196"/>
+      <c r="O29" s="179" t="s">
         <v>181</v>
       </c>
-      <c r="P29" s="103"/>
-      <c r="Q29" s="103"/>
-      <c r="R29" s="103"/>
-      <c r="S29" s="103"/>
-      <c r="T29" s="103"/>
-      <c r="U29" s="104"/>
-    </row>
-    <row r="30" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P29" s="179"/>
+      <c r="Q29" s="179"/>
+      <c r="R29" s="179"/>
+      <c r="S29" s="179"/>
+      <c r="T29" s="179"/>
+      <c r="U29" s="180"/>
+    </row>
+    <row r="30" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="49">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="B30" s="101" t="s">
+      <c r="B30" s="201" t="s">
         <v>182</v>
       </c>
-      <c r="C30" s="102"/>
-      <c r="D30" s="102"/>
-      <c r="E30" s="102"/>
-      <c r="F30" s="103" t="s">
+      <c r="C30" s="202"/>
+      <c r="D30" s="202"/>
+      <c r="E30" s="202"/>
+      <c r="F30" s="179" t="s">
         <v>183</v>
       </c>
-      <c r="G30" s="103"/>
-      <c r="H30" s="103"/>
-      <c r="I30" s="103"/>
-      <c r="J30" s="104"/>
-      <c r="K30" s="130" t="s">
+      <c r="G30" s="179"/>
+      <c r="H30" s="179"/>
+      <c r="I30" s="179"/>
+      <c r="J30" s="180"/>
+      <c r="K30" s="195" t="s">
         <v>184</v>
       </c>
-      <c r="L30" s="131"/>
-      <c r="M30" s="131"/>
-      <c r="N30" s="131"/>
-      <c r="O30" s="103">
+      <c r="L30" s="196"/>
+      <c r="M30" s="196"/>
+      <c r="N30" s="196"/>
+      <c r="O30" s="179">
         <v>100</v>
       </c>
-      <c r="P30" s="103"/>
-      <c r="Q30" s="103"/>
-      <c r="R30" s="103"/>
-      <c r="S30" s="103"/>
-      <c r="T30" s="103"/>
-      <c r="U30" s="104"/>
-    </row>
-    <row r="31" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="P30" s="179"/>
+      <c r="Q30" s="179"/>
+      <c r="R30" s="179"/>
+      <c r="S30" s="179"/>
+      <c r="T30" s="179"/>
+      <c r="U30" s="180"/>
+    </row>
+    <row r="31" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="49">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="B31" s="101" t="s">
+      <c r="B31" s="201" t="s">
         <v>185</v>
       </c>
-      <c r="C31" s="102"/>
-      <c r="D31" s="102"/>
-      <c r="E31" s="102"/>
-      <c r="F31" s="103" t="s">
+      <c r="C31" s="202"/>
+      <c r="D31" s="202"/>
+      <c r="E31" s="202"/>
+      <c r="F31" s="179" t="s">
         <v>186</v>
       </c>
-      <c r="G31" s="103"/>
-      <c r="H31" s="103"/>
-      <c r="I31" s="103"/>
-      <c r="J31" s="104"/>
-      <c r="K31" s="130" t="s">
+      <c r="G31" s="179"/>
+      <c r="H31" s="179"/>
+      <c r="I31" s="179"/>
+      <c r="J31" s="180"/>
+      <c r="K31" s="195" t="s">
         <v>187</v>
       </c>
-      <c r="L31" s="131"/>
-      <c r="M31" s="131"/>
-      <c r="N31" s="131"/>
-      <c r="O31" s="132" t="s">
+      <c r="L31" s="196"/>
+      <c r="M31" s="196"/>
+      <c r="N31" s="196"/>
+      <c r="O31" s="214" t="s">
         <v>188</v>
       </c>
-      <c r="P31" s="132"/>
-      <c r="Q31" s="132"/>
-      <c r="R31" s="132"/>
-      <c r="S31" s="132"/>
-      <c r="T31" s="132"/>
-      <c r="U31" s="133"/>
-    </row>
-    <row r="32" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="P31" s="214"/>
+      <c r="Q31" s="214"/>
+      <c r="R31" s="214"/>
+      <c r="S31" s="214"/>
+      <c r="T31" s="214"/>
+      <c r="U31" s="215"/>
+    </row>
+    <row r="32" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="49">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="B32" s="101" t="s">
+      <c r="B32" s="201" t="s">
         <v>189</v>
       </c>
-      <c r="C32" s="102"/>
-      <c r="D32" s="102"/>
-      <c r="E32" s="102"/>
-      <c r="F32" s="103" t="s">
+      <c r="C32" s="202"/>
+      <c r="D32" s="202"/>
+      <c r="E32" s="202"/>
+      <c r="F32" s="179" t="s">
         <v>190</v>
       </c>
-      <c r="G32" s="103"/>
-      <c r="H32" s="103"/>
-      <c r="I32" s="103"/>
-      <c r="J32" s="104"/>
-      <c r="K32" s="121"/>
-      <c r="L32" s="122"/>
-      <c r="M32" s="122"/>
-      <c r="N32" s="122"/>
-      <c r="O32" s="132"/>
-      <c r="P32" s="132"/>
-      <c r="Q32" s="132"/>
-      <c r="R32" s="132"/>
-      <c r="S32" s="132"/>
-      <c r="T32" s="132"/>
-      <c r="U32" s="133"/>
-    </row>
-    <row r="33" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="G32" s="179"/>
+      <c r="H32" s="179"/>
+      <c r="I32" s="179"/>
+      <c r="J32" s="180"/>
+      <c r="K32" s="205"/>
+      <c r="L32" s="206"/>
+      <c r="M32" s="206"/>
+      <c r="N32" s="206"/>
+      <c r="O32" s="214"/>
+      <c r="P32" s="214"/>
+      <c r="Q32" s="214"/>
+      <c r="R32" s="214"/>
+      <c r="S32" s="214"/>
+      <c r="T32" s="214"/>
+      <c r="U32" s="215"/>
+    </row>
+    <row r="33" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="49">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="B33" s="123" t="s">
+      <c r="B33" s="207" t="s">
         <v>191</v>
       </c>
-      <c r="C33" s="124"/>
-      <c r="D33" s="124"/>
-      <c r="E33" s="124"/>
-      <c r="F33" s="124"/>
-      <c r="G33" s="124"/>
-      <c r="H33" s="124"/>
-      <c r="I33" s="124"/>
-      <c r="J33" s="125"/>
-      <c r="K33" s="114" t="s">
+      <c r="C33" s="208"/>
+      <c r="D33" s="208"/>
+      <c r="E33" s="208"/>
+      <c r="F33" s="208"/>
+      <c r="G33" s="208"/>
+      <c r="H33" s="208"/>
+      <c r="I33" s="208"/>
+      <c r="J33" s="209"/>
+      <c r="K33" s="127" t="s">
         <v>192</v>
       </c>
-      <c r="L33" s="115"/>
-      <c r="M33" s="115"/>
-      <c r="N33" s="115"/>
-      <c r="O33" s="115"/>
-      <c r="P33" s="115"/>
-      <c r="Q33" s="115"/>
-      <c r="R33" s="115"/>
-      <c r="S33" s="115"/>
-      <c r="T33" s="115"/>
-      <c r="U33" s="116"/>
-    </row>
-    <row r="34" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L33" s="128"/>
+      <c r="M33" s="128"/>
+      <c r="N33" s="128"/>
+      <c r="O33" s="128"/>
+      <c r="P33" s="128"/>
+      <c r="Q33" s="128"/>
+      <c r="R33" s="128"/>
+      <c r="S33" s="128"/>
+      <c r="T33" s="128"/>
+      <c r="U33" s="129"/>
+    </row>
+    <row r="34" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="49">
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="B34" s="126" t="s">
+      <c r="B34" s="210" t="s">
         <v>193</v>
       </c>
-      <c r="C34" s="127"/>
-      <c r="D34" s="127"/>
-      <c r="E34" s="127"/>
-      <c r="F34" s="128" t="s">
+      <c r="C34" s="211"/>
+      <c r="D34" s="211"/>
+      <c r="E34" s="211"/>
+      <c r="F34" s="212" t="s">
         <v>194</v>
       </c>
-      <c r="G34" s="128"/>
-      <c r="H34" s="128"/>
-      <c r="I34" s="128"/>
-      <c r="J34" s="129"/>
+      <c r="G34" s="212"/>
+      <c r="H34" s="212"/>
+      <c r="I34" s="212"/>
+      <c r="J34" s="213"/>
       <c r="K34" s="70"/>
       <c r="L34" s="71"/>
       <c r="M34" s="71"/>
@@ -6667,24 +6670,24 @@
       <c r="T34" s="71"/>
       <c r="U34" s="72"/>
     </row>
-    <row r="35" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="49">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="B35" s="101" t="s">
+      <c r="B35" s="201" t="s">
         <v>195</v>
       </c>
-      <c r="C35" s="102"/>
-      <c r="D35" s="102"/>
-      <c r="E35" s="102"/>
-      <c r="F35" s="103" t="s">
+      <c r="C35" s="202"/>
+      <c r="D35" s="202"/>
+      <c r="E35" s="202"/>
+      <c r="F35" s="179" t="s">
         <v>196</v>
       </c>
-      <c r="G35" s="103"/>
-      <c r="H35" s="103"/>
-      <c r="I35" s="103"/>
-      <c r="J35" s="104"/>
+      <c r="G35" s="179"/>
+      <c r="H35" s="179"/>
+      <c r="I35" s="179"/>
+      <c r="J35" s="180"/>
       <c r="K35" s="70"/>
       <c r="L35" s="71"/>
       <c r="M35" s="71"/>
@@ -6697,24 +6700,24 @@
       <c r="T35" s="71"/>
       <c r="U35" s="72"/>
     </row>
-    <row r="36" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="49">
         <f t="shared" si="0"/>
         <v>33</v>
       </c>
-      <c r="B36" s="101" t="s">
+      <c r="B36" s="201" t="s">
         <v>197</v>
       </c>
-      <c r="C36" s="102"/>
-      <c r="D36" s="102"/>
-      <c r="E36" s="102"/>
-      <c r="F36" s="103" t="s">
+      <c r="C36" s="202"/>
+      <c r="D36" s="202"/>
+      <c r="E36" s="202"/>
+      <c r="F36" s="179" t="s">
         <v>198</v>
       </c>
-      <c r="G36" s="103"/>
-      <c r="H36" s="103"/>
-      <c r="I36" s="103"/>
-      <c r="J36" s="104"/>
+      <c r="G36" s="179"/>
+      <c r="H36" s="179"/>
+      <c r="I36" s="179"/>
+      <c r="J36" s="180"/>
       <c r="K36" s="70"/>
       <c r="L36" s="71"/>
       <c r="M36" s="71"/>
@@ -6727,24 +6730,24 @@
       <c r="T36" s="71"/>
       <c r="U36" s="72"/>
     </row>
-    <row r="37" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="49">
         <f t="shared" si="0"/>
         <v>34</v>
       </c>
-      <c r="B37" s="101" t="s">
+      <c r="B37" s="201" t="s">
         <v>199</v>
       </c>
-      <c r="C37" s="102"/>
-      <c r="D37" s="102"/>
-      <c r="E37" s="102"/>
-      <c r="F37" s="103" t="s">
+      <c r="C37" s="202"/>
+      <c r="D37" s="202"/>
+      <c r="E37" s="202"/>
+      <c r="F37" s="179" t="s">
         <v>90</v>
       </c>
-      <c r="G37" s="103"/>
-      <c r="H37" s="103"/>
-      <c r="I37" s="103"/>
-      <c r="J37" s="104"/>
+      <c r="G37" s="179"/>
+      <c r="H37" s="179"/>
+      <c r="I37" s="179"/>
+      <c r="J37" s="180"/>
       <c r="K37" s="70"/>
       <c r="L37" s="71"/>
       <c r="M37" s="71"/>
@@ -6757,24 +6760,24 @@
       <c r="T37" s="71"/>
       <c r="U37" s="72"/>
     </row>
-    <row r="38" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="49">
         <f t="shared" si="0"/>
         <v>35</v>
       </c>
-      <c r="B38" s="101" t="s">
+      <c r="B38" s="201" t="s">
         <v>200</v>
       </c>
-      <c r="C38" s="102"/>
-      <c r="D38" s="102"/>
-      <c r="E38" s="102"/>
-      <c r="F38" s="103" t="s">
+      <c r="C38" s="202"/>
+      <c r="D38" s="202"/>
+      <c r="E38" s="202"/>
+      <c r="F38" s="179" t="s">
         <v>201</v>
       </c>
-      <c r="G38" s="103"/>
-      <c r="H38" s="103"/>
-      <c r="I38" s="103"/>
-      <c r="J38" s="104"/>
+      <c r="G38" s="179"/>
+      <c r="H38" s="179"/>
+      <c r="I38" s="179"/>
+      <c r="J38" s="180"/>
       <c r="K38" s="70"/>
       <c r="L38" s="71"/>
       <c r="M38" s="71"/>
@@ -6787,24 +6790,24 @@
       <c r="T38" s="71"/>
       <c r="U38" s="72"/>
     </row>
-    <row r="39" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="49">
         <f t="shared" si="0"/>
         <v>36</v>
       </c>
-      <c r="B39" s="107" t="s">
+      <c r="B39" s="216" t="s">
         <v>202</v>
       </c>
-      <c r="C39" s="108"/>
-      <c r="D39" s="108"/>
-      <c r="E39" s="108"/>
-      <c r="F39" s="119" t="s">
+      <c r="C39" s="217"/>
+      <c r="D39" s="217"/>
+      <c r="E39" s="217"/>
+      <c r="F39" s="218" t="s">
         <v>194</v>
       </c>
-      <c r="G39" s="119"/>
-      <c r="H39" s="119"/>
-      <c r="I39" s="119"/>
-      <c r="J39" s="120"/>
+      <c r="G39" s="218"/>
+      <c r="H39" s="218"/>
+      <c r="I39" s="218"/>
+      <c r="J39" s="219"/>
       <c r="K39" s="70"/>
       <c r="L39" s="71"/>
       <c r="M39" s="71"/>
@@ -6817,22 +6820,22 @@
       <c r="T39" s="71"/>
       <c r="U39" s="72"/>
     </row>
-    <row r="40" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="49">
         <f t="shared" si="0"/>
         <v>37</v>
       </c>
-      <c r="B40" s="114" t="s">
+      <c r="B40" s="127" t="s">
         <v>203</v>
       </c>
-      <c r="C40" s="115"/>
-      <c r="D40" s="115"/>
-      <c r="E40" s="115"/>
-      <c r="F40" s="115"/>
-      <c r="G40" s="115"/>
-      <c r="H40" s="115"/>
-      <c r="I40" s="115"/>
-      <c r="J40" s="116"/>
+      <c r="C40" s="128"/>
+      <c r="D40" s="128"/>
+      <c r="E40" s="128"/>
+      <c r="F40" s="128"/>
+      <c r="G40" s="128"/>
+      <c r="H40" s="128"/>
+      <c r="I40" s="128"/>
+      <c r="J40" s="129"/>
       <c r="K40" s="70"/>
       <c r="L40" s="71"/>
       <c r="M40" s="71"/>
@@ -6845,24 +6848,24 @@
       <c r="T40" s="71"/>
       <c r="U40" s="72"/>
     </row>
-    <row r="41" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="49">
         <f t="shared" si="0"/>
         <v>38</v>
       </c>
-      <c r="B41" s="101" t="s">
+      <c r="B41" s="201" t="s">
         <v>204</v>
       </c>
-      <c r="C41" s="102"/>
-      <c r="D41" s="102"/>
-      <c r="E41" s="102"/>
-      <c r="F41" s="102"/>
-      <c r="G41" s="102"/>
-      <c r="H41" s="103" t="s">
+      <c r="C41" s="202"/>
+      <c r="D41" s="202"/>
+      <c r="E41" s="202"/>
+      <c r="F41" s="202"/>
+      <c r="G41" s="202"/>
+      <c r="H41" s="179" t="s">
         <v>205</v>
       </c>
-      <c r="I41" s="103"/>
-      <c r="J41" s="104"/>
+      <c r="I41" s="179"/>
+      <c r="J41" s="180"/>
       <c r="K41" s="70"/>
       <c r="L41" s="71"/>
       <c r="M41" s="71"/>
@@ -6875,24 +6878,24 @@
       <c r="T41" s="71"/>
       <c r="U41" s="72"/>
     </row>
-    <row r="42" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="49">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
-      <c r="B42" s="101" t="s">
+      <c r="B42" s="201" t="s">
         <v>206</v>
       </c>
-      <c r="C42" s="102"/>
-      <c r="D42" s="102"/>
-      <c r="E42" s="102"/>
-      <c r="F42" s="102"/>
-      <c r="G42" s="102"/>
-      <c r="H42" s="103" t="s">
+      <c r="C42" s="202"/>
+      <c r="D42" s="202"/>
+      <c r="E42" s="202"/>
+      <c r="F42" s="202"/>
+      <c r="G42" s="202"/>
+      <c r="H42" s="179" t="s">
         <v>207</v>
       </c>
-      <c r="I42" s="103"/>
-      <c r="J42" s="104"/>
+      <c r="I42" s="179"/>
+      <c r="J42" s="180"/>
       <c r="K42" s="70"/>
       <c r="L42" s="71"/>
       <c r="M42" s="71"/>
@@ -6905,199 +6908,335 @@
       <c r="T42" s="71"/>
       <c r="U42" s="72"/>
     </row>
-    <row r="43" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="49">
         <f t="shared" si="0"/>
         <v>40</v>
       </c>
-      <c r="B43" s="107" t="s">
+      <c r="B43" s="216" t="s">
         <v>208</v>
       </c>
-      <c r="C43" s="108"/>
-      <c r="D43" s="108"/>
-      <c r="E43" s="108"/>
-      <c r="F43" s="108"/>
-      <c r="G43" s="108"/>
-      <c r="H43" s="109" t="s">
+      <c r="C43" s="217"/>
+      <c r="D43" s="217"/>
+      <c r="E43" s="217"/>
+      <c r="F43" s="217"/>
+      <c r="G43" s="217"/>
+      <c r="H43" s="223" t="s">
         <v>209</v>
       </c>
-      <c r="I43" s="109"/>
-      <c r="J43" s="110"/>
-      <c r="K43" s="114" t="s">
+      <c r="I43" s="223"/>
+      <c r="J43" s="224"/>
+      <c r="K43" s="127" t="s">
         <v>210</v>
       </c>
-      <c r="L43" s="115"/>
-      <c r="M43" s="115"/>
-      <c r="N43" s="115"/>
-      <c r="O43" s="115"/>
-      <c r="P43" s="115"/>
-      <c r="Q43" s="115"/>
-      <c r="R43" s="115"/>
-      <c r="S43" s="115"/>
-      <c r="T43" s="115"/>
-      <c r="U43" s="116"/>
-    </row>
-    <row r="44" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="L43" s="128"/>
+      <c r="M43" s="128"/>
+      <c r="N43" s="128"/>
+      <c r="O43" s="128"/>
+      <c r="P43" s="128"/>
+      <c r="Q43" s="128"/>
+      <c r="R43" s="128"/>
+      <c r="S43" s="128"/>
+      <c r="T43" s="128"/>
+      <c r="U43" s="129"/>
+    </row>
+    <row r="44" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="49">
         <f t="shared" si="0"/>
         <v>41</v>
       </c>
-      <c r="B44" s="114" t="s">
+      <c r="B44" s="127" t="s">
         <v>211</v>
       </c>
-      <c r="C44" s="115"/>
-      <c r="D44" s="115"/>
-      <c r="E44" s="115"/>
-      <c r="F44" s="115"/>
-      <c r="G44" s="115"/>
-      <c r="H44" s="115"/>
-      <c r="I44" s="115"/>
-      <c r="J44" s="116"/>
+      <c r="C44" s="128"/>
+      <c r="D44" s="128"/>
+      <c r="E44" s="128"/>
+      <c r="F44" s="128"/>
+      <c r="G44" s="128"/>
+      <c r="H44" s="128"/>
+      <c r="I44" s="128"/>
+      <c r="J44" s="129"/>
       <c r="K44" s="52" t="s">
         <v>212</v>
       </c>
-      <c r="L44" s="105" t="s">
+      <c r="L44" s="221" t="s">
         <v>213</v>
       </c>
-      <c r="M44" s="105"/>
-      <c r="N44" s="105"/>
-      <c r="O44" s="105"/>
-      <c r="P44" s="105"/>
-      <c r="Q44" s="105"/>
-      <c r="R44" s="105"/>
-      <c r="S44" s="105"/>
-      <c r="T44" s="105"/>
-      <c r="U44" s="106"/>
-    </row>
-    <row r="45" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M44" s="221"/>
+      <c r="N44" s="221"/>
+      <c r="O44" s="221"/>
+      <c r="P44" s="221"/>
+      <c r="Q44" s="221"/>
+      <c r="R44" s="221"/>
+      <c r="S44" s="221"/>
+      <c r="T44" s="221"/>
+      <c r="U44" s="222"/>
+    </row>
+    <row r="45" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="49">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="B45" s="101" t="s">
+      <c r="B45" s="201" t="s">
         <v>214</v>
       </c>
-      <c r="C45" s="102"/>
-      <c r="D45" s="102"/>
-      <c r="E45" s="102"/>
-      <c r="F45" s="103" t="s">
+      <c r="C45" s="202"/>
+      <c r="D45" s="202"/>
+      <c r="E45" s="202"/>
+      <c r="F45" s="179" t="s">
         <v>215</v>
       </c>
-      <c r="G45" s="103"/>
-      <c r="H45" s="103"/>
-      <c r="I45" s="103"/>
-      <c r="J45" s="104"/>
+      <c r="G45" s="179"/>
+      <c r="H45" s="179"/>
+      <c r="I45" s="179"/>
+      <c r="J45" s="180"/>
       <c r="K45" s="53" t="s">
         <v>216</v>
       </c>
-      <c r="L45" s="117" t="s">
+      <c r="L45" s="227" t="s">
         <v>217</v>
       </c>
-      <c r="M45" s="117"/>
-      <c r="N45" s="117"/>
-      <c r="O45" s="117"/>
-      <c r="P45" s="117"/>
-      <c r="Q45" s="117"/>
-      <c r="R45" s="117"/>
-      <c r="S45" s="117"/>
-      <c r="T45" s="117"/>
-      <c r="U45" s="118"/>
-    </row>
-    <row r="46" spans="1:21" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M45" s="227"/>
+      <c r="N45" s="227"/>
+      <c r="O45" s="227"/>
+      <c r="P45" s="227"/>
+      <c r="Q45" s="227"/>
+      <c r="R45" s="227"/>
+      <c r="S45" s="227"/>
+      <c r="T45" s="227"/>
+      <c r="U45" s="228"/>
+    </row>
+    <row r="46" spans="1:21" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="49">
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="B46" s="101" t="s">
+      <c r="B46" s="201" t="s">
         <v>218</v>
       </c>
-      <c r="C46" s="102"/>
-      <c r="D46" s="102"/>
-      <c r="E46" s="102"/>
-      <c r="F46" s="103" t="s">
+      <c r="C46" s="202"/>
+      <c r="D46" s="202"/>
+      <c r="E46" s="202"/>
+      <c r="F46" s="179" t="s">
         <v>219</v>
       </c>
-      <c r="G46" s="103"/>
-      <c r="H46" s="103"/>
-      <c r="I46" s="103"/>
-      <c r="J46" s="104"/>
+      <c r="G46" s="179"/>
+      <c r="H46" s="179"/>
+      <c r="I46" s="179"/>
+      <c r="J46" s="180"/>
       <c r="K46" s="52" t="s">
         <v>220</v>
       </c>
-      <c r="L46" s="105" t="s">
+      <c r="L46" s="221" t="s">
         <v>221</v>
       </c>
-      <c r="M46" s="105"/>
-      <c r="N46" s="105"/>
-      <c r="O46" s="105"/>
-      <c r="P46" s="105"/>
-      <c r="Q46" s="105"/>
-      <c r="R46" s="105"/>
-      <c r="S46" s="105"/>
-      <c r="T46" s="105"/>
-      <c r="U46" s="106"/>
-    </row>
-    <row r="47" spans="1:21" ht="24.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M46" s="221"/>
+      <c r="N46" s="221"/>
+      <c r="O46" s="221"/>
+      <c r="P46" s="221"/>
+      <c r="Q46" s="221"/>
+      <c r="R46" s="221"/>
+      <c r="S46" s="221"/>
+      <c r="T46" s="221"/>
+      <c r="U46" s="222"/>
+    </row>
+    <row r="47" spans="1:21" ht="24.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A47" s="49">
         <f t="shared" si="0"/>
         <v>44</v>
       </c>
-      <c r="B47" s="107" t="s">
+      <c r="B47" s="216" t="s">
         <v>222</v>
       </c>
-      <c r="C47" s="108"/>
-      <c r="D47" s="108"/>
-      <c r="E47" s="108"/>
-      <c r="F47" s="109" t="s">
+      <c r="C47" s="217"/>
+      <c r="D47" s="217"/>
+      <c r="E47" s="217"/>
+      <c r="F47" s="223" t="s">
         <v>223</v>
       </c>
-      <c r="G47" s="109"/>
-      <c r="H47" s="109"/>
-      <c r="I47" s="109"/>
-      <c r="J47" s="110"/>
+      <c r="G47" s="223"/>
+      <c r="H47" s="223"/>
+      <c r="I47" s="223"/>
+      <c r="J47" s="224"/>
       <c r="K47" s="52" t="s">
         <v>224</v>
       </c>
-      <c r="L47" s="111" t="s">
+      <c r="L47" s="225" t="s">
         <v>225</v>
       </c>
-      <c r="M47" s="112"/>
-      <c r="N47" s="112"/>
-      <c r="O47" s="112"/>
-      <c r="P47" s="112"/>
-      <c r="Q47" s="112"/>
-      <c r="R47" s="112"/>
-      <c r="S47" s="112"/>
-      <c r="T47" s="112"/>
-      <c r="U47" s="113"/>
-    </row>
-    <row r="48" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="100" t="s">
+      <c r="M47" s="187"/>
+      <c r="N47" s="187"/>
+      <c r="O47" s="187"/>
+      <c r="P47" s="187"/>
+      <c r="Q47" s="187"/>
+      <c r="R47" s="187"/>
+      <c r="S47" s="187"/>
+      <c r="T47" s="187"/>
+      <c r="U47" s="226"/>
+    </row>
+    <row r="48" spans="1:21" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="220" t="s">
         <v>226</v>
       </c>
-      <c r="B48" s="100"/>
-      <c r="C48" s="100"/>
-      <c r="D48" s="100"/>
-      <c r="E48" s="100"/>
-      <c r="F48" s="100"/>
-      <c r="G48" s="100"/>
-      <c r="H48" s="100"/>
-      <c r="I48" s="100"/>
-      <c r="J48" s="100"/>
-      <c r="K48" s="100"/>
-      <c r="L48" s="100"/>
-      <c r="M48" s="100"/>
-      <c r="N48" s="100"/>
-      <c r="O48" s="100"/>
-      <c r="P48" s="100"/>
-      <c r="Q48" s="100"/>
-      <c r="R48" s="100"/>
-      <c r="S48" s="100"/>
-      <c r="T48" s="100"/>
-      <c r="U48" s="100"/>
+      <c r="B48" s="220"/>
+      <c r="C48" s="220"/>
+      <c r="D48" s="220"/>
+      <c r="E48" s="220"/>
+      <c r="F48" s="220"/>
+      <c r="G48" s="220"/>
+      <c r="H48" s="220"/>
+      <c r="I48" s="220"/>
+      <c r="J48" s="220"/>
+      <c r="K48" s="220"/>
+      <c r="L48" s="220"/>
+      <c r="M48" s="220"/>
+      <c r="N48" s="220"/>
+      <c r="O48" s="220"/>
+      <c r="P48" s="220"/>
+      <c r="Q48" s="220"/>
+      <c r="R48" s="220"/>
+      <c r="S48" s="220"/>
+      <c r="T48" s="220"/>
+      <c r="U48" s="220"/>
     </row>
   </sheetData>
   <mergeCells count="154">
+    <mergeCell ref="A48:U48"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="F46:J46"/>
+    <mergeCell ref="L46:U46"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="F47:J47"/>
+    <mergeCell ref="L47:U47"/>
+    <mergeCell ref="B43:G43"/>
+    <mergeCell ref="H43:J43"/>
+    <mergeCell ref="K43:U43"/>
+    <mergeCell ref="B44:J44"/>
+    <mergeCell ref="L44:U44"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="F45:J45"/>
+    <mergeCell ref="L45:U45"/>
+    <mergeCell ref="B39:E39"/>
+    <mergeCell ref="F39:J39"/>
+    <mergeCell ref="B40:J40"/>
+    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="H41:J41"/>
+    <mergeCell ref="B42:G42"/>
+    <mergeCell ref="H42:J42"/>
+    <mergeCell ref="B36:E36"/>
+    <mergeCell ref="F36:J36"/>
+    <mergeCell ref="B37:E37"/>
+    <mergeCell ref="F37:J37"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="F38:J38"/>
+    <mergeCell ref="K32:N32"/>
+    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="K33:U33"/>
+    <mergeCell ref="B34:E34"/>
+    <mergeCell ref="F34:J34"/>
+    <mergeCell ref="B35:E35"/>
+    <mergeCell ref="F35:J35"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="F30:J30"/>
+    <mergeCell ref="K30:N30"/>
+    <mergeCell ref="O30:U30"/>
+    <mergeCell ref="B31:E31"/>
+    <mergeCell ref="F31:J31"/>
+    <mergeCell ref="K31:N31"/>
+    <mergeCell ref="O31:U32"/>
+    <mergeCell ref="B32:E32"/>
+    <mergeCell ref="F32:J32"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="F28:J28"/>
+    <mergeCell ref="K28:N28"/>
+    <mergeCell ref="O28:U28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="F29:J29"/>
+    <mergeCell ref="K29:N29"/>
+    <mergeCell ref="O29:U29"/>
+    <mergeCell ref="B26:J26"/>
+    <mergeCell ref="K26:N26"/>
+    <mergeCell ref="O26:U26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="F27:J27"/>
+    <mergeCell ref="K27:N27"/>
+    <mergeCell ref="O27:U27"/>
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="K24:N24"/>
+    <mergeCell ref="O24:U24"/>
+    <mergeCell ref="B25:G25"/>
+    <mergeCell ref="H25:J25"/>
+    <mergeCell ref="K25:N25"/>
+    <mergeCell ref="O25:U25"/>
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="H22:J22"/>
+    <mergeCell ref="K22:U22"/>
+    <mergeCell ref="B23:G23"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="K23:N23"/>
+    <mergeCell ref="O23:U23"/>
+    <mergeCell ref="B21:G21"/>
+    <mergeCell ref="H21:J21"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="M21:N21"/>
+    <mergeCell ref="O21:Q21"/>
+    <mergeCell ref="R21:U21"/>
+    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="H20:J20"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="M20:N20"/>
+    <mergeCell ref="P20:Q20"/>
+    <mergeCell ref="R20:U20"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="P19:Q19"/>
+    <mergeCell ref="R19:U19"/>
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="R18:U18"/>
+    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="R17:U17"/>
+    <mergeCell ref="Q14:T14"/>
+    <mergeCell ref="B15:E15"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="H15:L15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:S15"/>
+    <mergeCell ref="T15:U15"/>
+    <mergeCell ref="L13:N13"/>
+    <mergeCell ref="O13:U13"/>
+    <mergeCell ref="B14:E14"/>
+    <mergeCell ref="G14:I14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="L14:N14"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="B16:J16"/>
+    <mergeCell ref="K16:U16"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="E13:G13"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="G7:J7"/>
+    <mergeCell ref="G8:J8"/>
+    <mergeCell ref="G9:J9"/>
+    <mergeCell ref="G10:J10"/>
+    <mergeCell ref="G11:J11"/>
+    <mergeCell ref="G12:J12"/>
     <mergeCell ref="A1:F3"/>
     <mergeCell ref="G1:O3"/>
     <mergeCell ref="P1:U1"/>
@@ -7116,160 +7255,24 @@
     <mergeCell ref="I5:L5"/>
     <mergeCell ref="M5:O5"/>
     <mergeCell ref="P5:U5"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B11:F11"/>
-    <mergeCell ref="B12:F12"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="E13:G13"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="G7:J7"/>
-    <mergeCell ref="G8:J8"/>
-    <mergeCell ref="G9:J9"/>
-    <mergeCell ref="G10:J10"/>
-    <mergeCell ref="G11:J11"/>
-    <mergeCell ref="G12:J12"/>
-    <mergeCell ref="L13:N13"/>
-    <mergeCell ref="O13:U13"/>
-    <mergeCell ref="B14:E14"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="L14:N14"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="B16:J16"/>
-    <mergeCell ref="K16:U16"/>
-    <mergeCell ref="B17:G17"/>
-    <mergeCell ref="H17:J17"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="P17:Q17"/>
-    <mergeCell ref="R17:U17"/>
-    <mergeCell ref="Q14:T14"/>
-    <mergeCell ref="B15:E15"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="H15:L15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:S15"/>
-    <mergeCell ref="T15:U15"/>
-    <mergeCell ref="B19:G19"/>
-    <mergeCell ref="H19:J19"/>
-    <mergeCell ref="K19:L19"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="P19:Q19"/>
-    <mergeCell ref="R19:U19"/>
-    <mergeCell ref="B18:G18"/>
-    <mergeCell ref="H18:J18"/>
-    <mergeCell ref="K18:L18"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="R18:U18"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="H21:J21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="M21:N21"/>
-    <mergeCell ref="O21:Q21"/>
-    <mergeCell ref="R21:U21"/>
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="H20:J20"/>
-    <mergeCell ref="K20:L20"/>
-    <mergeCell ref="M20:N20"/>
-    <mergeCell ref="P20:Q20"/>
-    <mergeCell ref="R20:U20"/>
-    <mergeCell ref="B24:G24"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="K24:N24"/>
-    <mergeCell ref="O24:U24"/>
-    <mergeCell ref="B25:G25"/>
-    <mergeCell ref="H25:J25"/>
-    <mergeCell ref="K25:N25"/>
-    <mergeCell ref="O25:U25"/>
-    <mergeCell ref="B22:G22"/>
-    <mergeCell ref="H22:J22"/>
-    <mergeCell ref="K22:U22"/>
-    <mergeCell ref="B23:G23"/>
-    <mergeCell ref="H23:J23"/>
-    <mergeCell ref="K23:N23"/>
-    <mergeCell ref="O23:U23"/>
-    <mergeCell ref="B28:E28"/>
-    <mergeCell ref="F28:J28"/>
-    <mergeCell ref="K28:N28"/>
-    <mergeCell ref="O28:U28"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="F29:J29"/>
-    <mergeCell ref="K29:N29"/>
-    <mergeCell ref="O29:U29"/>
-    <mergeCell ref="B26:J26"/>
-    <mergeCell ref="K26:N26"/>
-    <mergeCell ref="O26:U26"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="F27:J27"/>
-    <mergeCell ref="K27:N27"/>
-    <mergeCell ref="O27:U27"/>
-    <mergeCell ref="K32:N32"/>
-    <mergeCell ref="B33:J33"/>
-    <mergeCell ref="K33:U33"/>
-    <mergeCell ref="B34:E34"/>
-    <mergeCell ref="F34:J34"/>
-    <mergeCell ref="B35:E35"/>
-    <mergeCell ref="F35:J35"/>
-    <mergeCell ref="B30:E30"/>
-    <mergeCell ref="F30:J30"/>
-    <mergeCell ref="K30:N30"/>
-    <mergeCell ref="O30:U30"/>
-    <mergeCell ref="B31:E31"/>
-    <mergeCell ref="F31:J31"/>
-    <mergeCell ref="K31:N31"/>
-    <mergeCell ref="O31:U32"/>
-    <mergeCell ref="B32:E32"/>
-    <mergeCell ref="F32:J32"/>
-    <mergeCell ref="B39:E39"/>
-    <mergeCell ref="F39:J39"/>
-    <mergeCell ref="B40:J40"/>
-    <mergeCell ref="B41:G41"/>
-    <mergeCell ref="H41:J41"/>
-    <mergeCell ref="B42:G42"/>
-    <mergeCell ref="H42:J42"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="F36:J36"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="F37:J37"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="F38:J38"/>
-    <mergeCell ref="A48:U48"/>
-    <mergeCell ref="B46:E46"/>
-    <mergeCell ref="F46:J46"/>
-    <mergeCell ref="L46:U46"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="F47:J47"/>
-    <mergeCell ref="L47:U47"/>
-    <mergeCell ref="B43:G43"/>
-    <mergeCell ref="H43:J43"/>
-    <mergeCell ref="K43:U43"/>
-    <mergeCell ref="B44:J44"/>
-    <mergeCell ref="L44:U44"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="F45:J45"/>
-    <mergeCell ref="L45:U45"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.5" bottom="0.5" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="65" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="62" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF4500"/>
   </sheetPr>
   <dimension ref="A10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="10" spans="1:1" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" ht="24.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="87" t="s">
         <v>262</v>
       </c>

</xml_diff>